<commit_message>
updated files and analysis for NPH correction off
</commit_message>
<xml_diff>
--- a/data/Czech/KCOR_summary.xlsx
+++ b/data/Czech/KCOR_summary.xlsx
@@ -493,17 +493,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1.3097</t>
+          <t>1.2730</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.281</t>
+          <t>1.245</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.339</t>
+          <t>1.302</t>
         </is>
       </c>
     </row>
@@ -516,17 +516,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.9837</t>
+          <t>0.9372</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.902</t>
+          <t>0.860</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.073</t>
+          <t>1.021</t>
         </is>
       </c>
     </row>
@@ -539,17 +539,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1.0525</t>
+          <t>1.0132</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>1.008</t>
+          <t>0.971</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.099</t>
+          <t>1.057</t>
         </is>
       </c>
     </row>
@@ -562,17 +562,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1.5883</t>
+          <t>1.5400</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.539</t>
+          <t>1.492</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.639</t>
+          <t>1.589</t>
         </is>
       </c>
     </row>
@@ -585,17 +585,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1.6341</t>
+          <t>1.6034</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.511</t>
+          <t>1.482</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.768</t>
+          <t>1.734</t>
         </is>
       </c>
     </row>
@@ -608,17 +608,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.4582</t>
+          <t>1.4221</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.264</t>
+          <t>1.232</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.683</t>
+          <t>1.641</t>
         </is>
       </c>
     </row>
@@ -631,17 +631,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>3.0768</t>
+          <t>2.9826</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.415</t>
+          <t>2.341</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.920</t>
+          <t>3.800</t>
         </is>
       </c>
     </row>
@@ -654,17 +654,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.0891</t>
+          <t>1.0472</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.719</t>
+          <t>0.691</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.650</t>
+          <t>1.586</t>
         </is>
       </c>
     </row>
@@ -677,17 +677,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.6680</t>
+          <t>2.5682</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.694</t>
+          <t>1.632</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>4.203</t>
+          <t>4.041</t>
         </is>
       </c>
     </row>
@@ -700,17 +700,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12.6258</t>
+          <t>12.4845</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5.940</t>
+          <t>5.875</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>26.839</t>
+          <t>26.530</t>
         </is>
       </c>
     </row>
@@ -741,17 +741,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1.5778</t>
+          <t>1.5337</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.552</t>
+          <t>1.508</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.604</t>
+          <t>1.559</t>
         </is>
       </c>
     </row>
@@ -764,17 +764,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1.3491</t>
+          <t>1.2853</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.290</t>
+          <t>1.230</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.411</t>
+          <t>1.343</t>
         </is>
       </c>
     </row>
@@ -787,17 +787,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.5714</t>
+          <t>1.5126</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.531</t>
+          <t>1.474</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.613</t>
+          <t>1.552</t>
         </is>
       </c>
     </row>
@@ -810,17 +810,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1.6561</t>
+          <t>1.6057</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.593</t>
+          <t>1.545</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.722</t>
+          <t>1.669</t>
         </is>
       </c>
     </row>
@@ -833,17 +833,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1.2616</t>
+          <t>1.2380</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.171</t>
+          <t>1.149</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.360</t>
+          <t>1.334</t>
         </is>
       </c>
     </row>
@@ -856,17 +856,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.2856</t>
+          <t>1.2537</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.111</t>
+          <t>1.083</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.488</t>
+          <t>1.451</t>
         </is>
       </c>
     </row>
@@ -879,17 +879,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.1379</t>
+          <t>1.1030</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.895</t>
+          <t>0.868</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.446</t>
+          <t>1.402</t>
         </is>
       </c>
     </row>
@@ -902,17 +902,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.6223</t>
+          <t>0.5983</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.403</t>
+          <t>0.388</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0.961</t>
+          <t>0.924</t>
         </is>
       </c>
     </row>
@@ -925,17 +925,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1.2343</t>
+          <t>1.1881</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.736</t>
+          <t>0.709</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2.070</t>
+          <t>1.991</t>
         </is>
       </c>
     </row>
@@ -948,17 +948,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2.2733</t>
+          <t>2.2478</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.319</t>
+          <t>0.315</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>16.215</t>
+          <t>16.031</t>
         </is>
       </c>
     </row>
@@ -1289,17 +1289,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1.1975</t>
+          <t>1.1573</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.175</t>
+          <t>1.135</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.221</t>
+          <t>1.180</t>
         </is>
       </c>
     </row>
@@ -1312,17 +1312,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.7004</t>
+          <t>0.6681</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.633</t>
+          <t>0.604</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.775</t>
+          <t>0.739</t>
         </is>
       </c>
     </row>
@@ -1335,17 +1335,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1.0274</t>
+          <t>0.9813</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.977</t>
+          <t>0.933</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.081</t>
+          <t>1.032</t>
         </is>
       </c>
     </row>
@@ -1358,17 +1358,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1.1094</t>
+          <t>1.0733</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.072</t>
+          <t>1.038</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.148</t>
+          <t>1.110</t>
         </is>
       </c>
     </row>
@@ -1381,17 +1381,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1.5367</t>
+          <t>1.4924</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.485</t>
+          <t>1.442</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.590</t>
+          <t>1.544</t>
         </is>
       </c>
     </row>
@@ -1404,17 +1404,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.4665</t>
+          <t>1.4221</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.379</t>
+          <t>1.338</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.559</t>
+          <t>1.511</t>
         </is>
       </c>
     </row>
@@ -1427,17 +1427,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1.2574</t>
+          <t>1.2246</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.118</t>
+          <t>1.089</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.414</t>
+          <t>1.377</t>
         </is>
       </c>
     </row>
@@ -1450,17 +1450,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.2937</t>
+          <t>1.2424</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.031</t>
+          <t>0.991</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.624</t>
+          <t>1.558</t>
         </is>
       </c>
     </row>
@@ -1473,17 +1473,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.1189</t>
+          <t>1.0686</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.691</t>
+          <t>0.661</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.811</t>
+          <t>1.728</t>
         </is>
       </c>
     </row>
@@ -1496,17 +1496,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12.0943</t>
+          <t>11.9909</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>8.251</t>
+          <t>8.184</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>17.728</t>
+          <t>17.569</t>
         </is>
       </c>
     </row>
@@ -1537,17 +1537,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1.1422</t>
+          <t>1.1039</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.126</t>
+          <t>1.089</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.159</t>
+          <t>1.120</t>
         </is>
       </c>
     </row>
@@ -1560,17 +1560,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.9643</t>
+          <t>0.9198</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.923</t>
+          <t>0.882</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.007</t>
+          <t>0.959</t>
         </is>
       </c>
     </row>
@@ -1583,17 +1583,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.0574</t>
+          <t>1.0100</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.031</t>
+          <t>0.986</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.084</t>
+          <t>1.035</t>
         </is>
       </c>
     </row>
@@ -1606,17 +1606,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1.2979</t>
+          <t>1.2556</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.265</t>
+          <t>1.224</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.332</t>
+          <t>1.288</t>
         </is>
       </c>
     </row>
@@ -1629,17 +1629,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1.1010</t>
+          <t>1.0692</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.047</t>
+          <t>1.017</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.158</t>
+          <t>1.124</t>
         </is>
       </c>
     </row>
@@ -1652,17 +1652,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.2918</t>
+          <t>1.2528</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.177</t>
+          <t>1.142</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.418</t>
+          <t>1.375</t>
         </is>
       </c>
     </row>
@@ -1675,17 +1675,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.0577</t>
+          <t>1.0301</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.911</t>
+          <t>0.888</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.228</t>
+          <t>1.195</t>
         </is>
       </c>
     </row>
@@ -1698,17 +1698,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2.8176</t>
+          <t>2.7059</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.202</t>
+          <t>2.116</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3.605</t>
+          <t>3.460</t>
         </is>
       </c>
     </row>
@@ -1721,17 +1721,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.9244</t>
+          <t>0.8828</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.664</t>
+          <t>0.635</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.287</t>
+          <t>1.227</t>
         </is>
       </c>
     </row>
@@ -1744,17 +1744,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>7.1546</t>
+          <t>7.0935</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3.793</t>
+          <t>3.762</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>13.495</t>
+          <t>13.377</t>
         </is>
       </c>
     </row>
@@ -2085,17 +2085,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.9653</t>
+          <t>0.9292</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.944</t>
+          <t>0.909</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.987</t>
+          <t>0.950</t>
         </is>
       </c>
     </row>
@@ -2108,17 +2108,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.6673</t>
+          <t>0.6358</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.593</t>
+          <t>0.565</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.751</t>
+          <t>0.715</t>
         </is>
       </c>
     </row>
@@ -2131,17 +2131,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.9209</t>
+          <t>0.8751</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.871</t>
+          <t>0.828</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.973</t>
+          <t>0.924</t>
         </is>
       </c>
     </row>
@@ -2154,17 +2154,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.8833</t>
+          <t>0.8511</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.846</t>
+          <t>0.815</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.923</t>
+          <t>0.889</t>
         </is>
       </c>
     </row>
@@ -2177,17 +2177,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1.1270</t>
+          <t>1.0902</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.082</t>
+          <t>1.047</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.174</t>
+          <t>1.135</t>
         </is>
       </c>
     </row>
@@ -2200,17 +2200,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.1444</t>
+          <t>1.1077</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.079</t>
+          <t>1.045</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.214</t>
+          <t>1.175</t>
         </is>
       </c>
     </row>
@@ -2223,17 +2223,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1.2772</t>
+          <t>1.2436</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.168</t>
+          <t>1.138</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.397</t>
+          <t>1.359</t>
         </is>
       </c>
     </row>
@@ -2246,17 +2246,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.9802</t>
+          <t>0.9481</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.823</t>
+          <t>0.797</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.168</t>
+          <t>1.128</t>
         </is>
       </c>
     </row>
@@ -2269,17 +2269,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.3550</t>
+          <t>3.1828</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2.392</t>
+          <t>2.274</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>4.707</t>
+          <t>4.455</t>
         </is>
       </c>
     </row>
@@ -2292,17 +2292,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.5925</t>
+          <t>0.5841</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.305</t>
+          <t>0.300</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.152</t>
+          <t>1.135</t>
         </is>
       </c>
     </row>
@@ -2333,17 +2333,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1.0567</t>
+          <t>1.0172</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.043</t>
+          <t>1.004</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.071</t>
+          <t>1.031</t>
         </is>
       </c>
     </row>
@@ -2356,17 +2356,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.8816</t>
+          <t>0.8401</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.844</t>
+          <t>0.805</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0.921</t>
+          <t>0.876</t>
         </is>
       </c>
     </row>
@@ -2379,17 +2379,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.9856</t>
+          <t>0.9366</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.961</t>
+          <t>0.914</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.011</t>
+          <t>0.960</t>
         </is>
       </c>
     </row>
@@ -2402,17 +2402,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1.0860</t>
+          <t>1.0464</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.060</t>
+          <t>1.022</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.113</t>
+          <t>1.071</t>
         </is>
       </c>
     </row>
@@ -2425,17 +2425,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1.3357</t>
+          <t>1.2922</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.291</t>
+          <t>1.249</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.382</t>
+          <t>1.337</t>
         </is>
       </c>
     </row>
@@ -2448,17 +2448,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.0912</t>
+          <t>1.0562</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.018</t>
+          <t>0.986</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.169</t>
+          <t>1.131</t>
         </is>
       </c>
     </row>
@@ -2471,17 +2471,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.1486</t>
+          <t>1.1184</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1.026</t>
+          <t>0.999</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.286</t>
+          <t>1.252</t>
         </is>
       </c>
     </row>
@@ -2494,17 +2494,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.3253</t>
+          <t>1.2819</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.082</t>
+          <t>1.048</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.623</t>
+          <t>1.568</t>
         </is>
       </c>
     </row>
@@ -2517,17 +2517,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2.2608</t>
+          <t>2.1448</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1.683</t>
+          <t>1.600</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>3.038</t>
+          <t>2.875</t>
         </is>
       </c>
     </row>
@@ -2540,17 +2540,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1.3854</t>
+          <t>1.3659</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.968</t>
+          <t>0.955</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.984</t>
+          <t>1.954</t>
         </is>
       </c>
     </row>
@@ -2881,17 +2881,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.6494</t>
+          <t>0.6229</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.626</t>
+          <t>0.601</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.674</t>
+          <t>0.646</t>
         </is>
       </c>
     </row>
@@ -2904,17 +2904,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.4475</t>
+          <t>0.4255</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.373</t>
+          <t>0.354</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.537</t>
+          <t>0.511</t>
         </is>
       </c>
     </row>
@@ -2927,17 +2927,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.6207</t>
+          <t>0.5884</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.572</t>
+          <t>0.542</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.674</t>
+          <t>0.638</t>
         </is>
       </c>
     </row>
@@ -2950,17 +2950,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.6032</t>
+          <t>0.5786</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.562</t>
+          <t>0.540</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.647</t>
+          <t>0.620</t>
         </is>
       </c>
     </row>
@@ -2973,17 +2973,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.6362</t>
+          <t>0.6146</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.590</t>
+          <t>0.570</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.686</t>
+          <t>0.662</t>
         </is>
       </c>
     </row>
@@ -2996,17 +2996,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.9824</t>
+          <t>0.9494</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.880</t>
+          <t>0.850</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.097</t>
+          <t>1.060</t>
         </is>
       </c>
     </row>
@@ -3019,17 +3019,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1.0974</t>
+          <t>1.0622</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.947</t>
+          <t>0.917</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.272</t>
+          <t>1.230</t>
         </is>
       </c>
     </row>
@@ -3042,17 +3042,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.2513</t>
+          <t>1.2058</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.027</t>
+          <t>0.990</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.525</t>
+          <t>1.468</t>
         </is>
       </c>
     </row>
@@ -3065,17 +3065,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.0556</t>
+          <t>1.0090</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.770</t>
+          <t>0.738</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.446</t>
+          <t>1.379</t>
         </is>
       </c>
     </row>
@@ -3088,17 +3088,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.2004</t>
+          <t>1.1597</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.815</t>
+          <t>0.789</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.767</t>
+          <t>1.704</t>
         </is>
       </c>
     </row>
@@ -3129,17 +3129,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.9110</t>
+          <t>0.8737</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.900</t>
+          <t>0.863</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0.923</t>
+          <t>0.885</t>
         </is>
       </c>
     </row>
@@ -3152,17 +3152,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.7837</t>
+          <t>0.7453</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.751</t>
+          <t>0.715</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0.818</t>
+          <t>0.777</t>
         </is>
       </c>
     </row>
@@ -3175,17 +3175,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.8268</t>
+          <t>0.7838</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.807</t>
+          <t>0.765</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0.848</t>
+          <t>0.803</t>
         </is>
       </c>
     </row>
@@ -3198,17 +3198,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.9152</t>
+          <t>0.8780</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.894</t>
+          <t>0.858</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0.937</t>
+          <t>0.898</t>
         </is>
       </c>
     </row>
@@ -3221,17 +3221,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.9469</t>
+          <t>0.9147</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.919</t>
+          <t>0.888</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0.976</t>
+          <t>0.942</t>
         </is>
       </c>
     </row>
@@ -3244,17 +3244,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.3073</t>
+          <t>1.2633</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.244</t>
+          <t>1.203</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.374</t>
+          <t>1.327</t>
         </is>
       </c>
     </row>
@@ -3267,17 +3267,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.1390</t>
+          <t>1.1025</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1.054</t>
+          <t>1.022</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.230</t>
+          <t>1.190</t>
         </is>
       </c>
     </row>
@@ -3290,17 +3290,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.6839</t>
+          <t>1.6227</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.460</t>
+          <t>1.410</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.942</t>
+          <t>1.868</t>
         </is>
       </c>
     </row>
@@ -3313,17 +3313,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1.1717</t>
+          <t>1.1200</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.919</t>
+          <t>0.881</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.495</t>
+          <t>1.424</t>
         </is>
       </c>
     </row>
@@ -3336,17 +3336,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.2940</t>
+          <t>0.2840</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.188</t>
+          <t>0.182</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0.460</t>
+          <t>0.444</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
v7.5 with infufficent data fix
</commit_message>
<xml_diff>
--- a/data/Czech/KCOR_summary.xlsx
+++ b/data/Czech/KCOR_summary.xlsx
@@ -827,17 +827,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.0309</t>
+          <t>1.0730</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.676</t>
+          <t>0.703</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.572</t>
+          <t>1.637</t>
         </is>
       </c>
       <c r="F11" t="b">
@@ -847,7 +847,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>99.99836701224508</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
         <v>11</v>
@@ -1271,27 +1271,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.6115</t>
+          <t>0.6223</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.401</t>
+          <t>0.403</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0.932</t>
+          <t>0.961</t>
         </is>
       </c>
       <c r="F23" t="b">
         <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>67.15278858582882</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>99.99836701224508</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
         <v>11</v>
@@ -1715,24 +1715,24 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>0.5932</t>
+          <t>0.5799</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>0.329</t>
+          <t>0.319</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.070</t>
+          <t>1.056</t>
         </is>
       </c>
       <c r="F35" t="b">
         <v>1</v>
       </c>
       <c r="G35" t="n">
-        <v>67.15278858582882</v>
+        <v>0</v>
       </c>
       <c r="H35" t="n">
         <v>0</v>
@@ -2249,24 +2249,24 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.2015</t>
+          <t>1.1890</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.946</t>
+          <t>0.934</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.525</t>
+          <t>1.513</t>
         </is>
       </c>
       <c r="F11" t="b">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>20.17276949813065</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
         <v>59.757586912448</v>
@@ -3137,17 +3137,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>2.2885</t>
+          <t>2.3124</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1.645</t>
+          <t>1.659</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>3.184</t>
+          <t>3.223</t>
         </is>
       </c>
       <c r="F35" t="b">
@@ -3157,7 +3157,7 @@
         <v>3.072968489481465e-05</v>
       </c>
       <c r="H35" t="n">
-        <v>20.17276949813065</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>11</v>
@@ -3425,27 +3425,27 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.7458</t>
+          <t>0.7689</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.667</t>
+          <t>0.682</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.834</t>
+          <t>0.867</t>
         </is>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>0.368184590370468</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>0.4381125719082086</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
         <v>11</v>
@@ -3671,27 +3671,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>0.9494</t>
+          <t>0.9988</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.798</t>
+          <t>0.838</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.130</t>
+          <t>1.191</t>
         </is>
       </c>
       <c r="F11" t="b">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>0.004735882525673585</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>99.99999874596539</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
         <v>11</v>
@@ -3712,17 +3712,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.2920</t>
+          <t>3.3550</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2.349</t>
+          <t>2.392</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>4.614</t>
+          <t>4.707</t>
         </is>
       </c>
       <c r="F12" t="b">
@@ -3732,7 +3732,7 @@
         <v>0.0002366379193354806</v>
       </c>
       <c r="H12" t="n">
-        <v>99.98397501305337</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
         <v>11</v>
@@ -3869,17 +3869,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.9351</t>
+          <t>1.0158</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.894</t>
+          <t>0.969</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0.978</t>
+          <t>1.065</t>
         </is>
       </c>
       <c r="F17" t="b">
@@ -3889,7 +3889,7 @@
         <v>1e-10</v>
       </c>
       <c r="H17" t="n">
-        <v>0.4381125719082086</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
         <v>11</v>
@@ -4115,17 +4115,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.2836</t>
+          <t>1.3504</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.049</t>
+          <t>1.102</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.570</t>
+          <t>1.655</t>
         </is>
       </c>
       <c r="F23" t="b">
@@ -4135,7 +4135,7 @@
         <v>0.000434689012210665</v>
       </c>
       <c r="H23" t="n">
-        <v>99.99999874596539</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
         <v>11</v>
@@ -4156,17 +4156,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2.0579</t>
+          <t>2.0973</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1.501</t>
+          <t>1.528</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2.822</t>
+          <t>2.879</t>
         </is>
       </c>
       <c r="F24" t="b">
@@ -4176,7 +4176,7 @@
         <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>99.98397501305337</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
         <v>11</v>
@@ -4313,17 +4313,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1.2538</t>
+          <t>1.3212</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1.122</t>
+          <t>1.175</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.401</t>
+          <t>1.486</t>
         </is>
       </c>
       <c r="F29" t="b">
@@ -4333,7 +4333,7 @@
         <v>1e-10</v>
       </c>
       <c r="H29" t="n">
-        <v>0.368184590370468</v>
+        <v>0</v>
       </c>
       <c r="I29" t="n">
         <v>11</v>
@@ -4579,7 +4579,7 @@
         <v>0.000434689012210665</v>
       </c>
       <c r="H35" t="n">
-        <v>0.004735882525673585</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>11</v>
@@ -4847,17 +4847,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.6070</t>
+          <t>0.6624</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.528</t>
+          <t>0.575</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.698</t>
+          <t>0.763</t>
         </is>
       </c>
       <c r="F5" t="b">
@@ -4867,7 +4867,7 @@
         <v>1.387534855497648</v>
       </c>
       <c r="H5" t="n">
-        <v>0.4537941446299353</v>
+        <v>0</v>
       </c>
       <c r="I5" t="n">
         <v>5</v>
@@ -4929,24 +4929,24 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.6865</t>
+          <t>0.6087</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.644</t>
+          <t>0.565</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.732</t>
+          <t>0.655</t>
         </is>
       </c>
       <c r="F7" t="b">
         <v>1</v>
       </c>
       <c r="G7" t="n">
-        <v>5.144869335656168</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
         <v>2.979749884865235</v>
@@ -4970,24 +4970,24 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.7166</t>
+          <t>0.6358</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.669</t>
+          <t>0.588</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.767</t>
+          <t>0.687</t>
         </is>
       </c>
       <c r="F8" t="b">
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>12.94399970085989</v>
+        <v>0</v>
       </c>
       <c r="H8" t="n">
         <v>7.652980279154328</v>
@@ -5093,27 +5093,27 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.1542</t>
+          <t>1.2151</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.940</t>
+          <t>0.986</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.417</t>
+          <t>1.497</t>
         </is>
       </c>
       <c r="F11" t="b">
         <v>1</v>
       </c>
       <c r="G11" t="n">
-        <v>18.07141117982593</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>99.99832749090832</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
         <v>5</v>
@@ -5134,27 +5134,27 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.0486</t>
+          <t>1.0614</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.769</t>
+          <t>0.774</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.430</t>
+          <t>1.455</t>
         </is>
       </c>
       <c r="F12" t="b">
         <v>1</v>
       </c>
       <c r="G12" t="n">
-        <v>99.99883438093936</v>
+        <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>99.99655614702037</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
         <v>5</v>
@@ -5175,17 +5175,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.2080</t>
+          <t>1.2225</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.820</t>
+          <t>0.829</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.779</t>
+          <t>1.802</t>
         </is>
       </c>
       <c r="F13" t="b">
@@ -5195,7 +5195,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>99.88585064778931</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
         <v>5</v>
@@ -5291,17 +5291,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.8453</t>
+          <t>0.9224</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.808</t>
+          <t>0.880</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0.884</t>
+          <t>0.967</t>
         </is>
       </c>
       <c r="F17" t="b">
@@ -5311,7 +5311,7 @@
         <v>1e-10</v>
       </c>
       <c r="H17" t="n">
-        <v>0.4537941446299353</v>
+        <v>0</v>
       </c>
       <c r="I17" t="n">
         <v>5</v>
@@ -5537,17 +5537,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.6230</t>
+          <t>1.7184</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.410</t>
+          <t>1.489</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.868</t>
+          <t>1.983</t>
         </is>
       </c>
       <c r="F23" t="b">
@@ -5557,7 +5557,7 @@
         <v>0.001600423735280132</v>
       </c>
       <c r="H23" t="n">
-        <v>99.99832749090832</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
         <v>5</v>
@@ -5566,7 +5566,7 @@
         <v>5</v>
       </c>
       <c r="K23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -5578,27 +5578,27 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1.1687</t>
+          <t>1.1782</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.920</t>
+          <t>0.923</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.484</t>
+          <t>1.503</t>
         </is>
       </c>
       <c r="F24" t="b">
         <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>73.33347320005834</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>99.99655614702037</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
         <v>5</v>
@@ -5619,17 +5619,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.2685</t>
+          <t>0.2717</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.160</t>
+          <t>0.162</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0.450</t>
+          <t>0.456</t>
         </is>
       </c>
       <c r="F25" t="b">
@@ -5639,7 +5639,7 @@
         <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>99.88585064778931</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
         <v>5</v>
@@ -5817,17 +5817,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1.4057</t>
+          <t>1.5854</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>1.319</t>
+          <t>1.473</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.498</t>
+          <t>1.706</t>
         </is>
       </c>
       <c r="F31" t="b">
@@ -5837,7 +5837,7 @@
         <v>3.023117197968237e-09</v>
       </c>
       <c r="H31" t="n">
-        <v>5.144869335656168</v>
+        <v>0</v>
       </c>
       <c r="I31" t="n">
         <v>5</v>
@@ -5858,17 +5858,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>1.3639</t>
+          <t>1.5373</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>1.274</t>
+          <t>1.422</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>1.461</t>
+          <t>1.662</t>
         </is>
       </c>
       <c r="F32" t="b">
@@ -5878,7 +5878,7 @@
         <v>1e-10</v>
       </c>
       <c r="H32" t="n">
-        <v>12.94399970085989</v>
+        <v>0</v>
       </c>
       <c r="I32" t="n">
         <v>5</v>
@@ -5981,17 +5981,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1.4061</t>
+          <t>1.4142</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1.121</t>
+          <t>1.126</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.764</t>
+          <t>1.776</t>
         </is>
       </c>
       <c r="F35" t="b">
@@ -6001,7 +6001,7 @@
         <v>0.001600423735280132</v>
       </c>
       <c r="H35" t="n">
-        <v>18.07141117982593</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>5</v>
@@ -6022,27 +6022,27 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1.1145</t>
+          <t>1.1100</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>0.785</t>
+          <t>0.777</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.583</t>
+          <t>1.585</t>
         </is>
       </c>
       <c r="F36" t="b">
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>73.33347320005834</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>99.99883438093936</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
         <v>5</v>
@@ -6269,24 +6269,24 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.9217</t>
+          <t>0.8713</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.708</t>
+          <t>0.657</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.200</t>
+          <t>1.155</t>
         </is>
       </c>
       <c r="F5" t="b">
         <v>1</v>
       </c>
       <c r="G5" t="n">
-        <v>0.4324265093155894</v>
+        <v>0</v>
       </c>
       <c r="H5" t="n">
         <v>1.483209665604275</v>
@@ -6433,24 +6433,24 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.8509</t>
+          <t>0.6965</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.726</t>
+          <t>0.570</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0.997</t>
+          <t>0.851</t>
         </is>
       </c>
       <c r="F9" t="b">
         <v>1</v>
       </c>
       <c r="G9" t="n">
-        <v>27.49288398547458</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
         <v>30.03019045477097</v>
@@ -6474,27 +6474,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.9792</t>
+          <t>0.9082</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.807</t>
+          <t>0.704</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.188</t>
+          <t>1.171</t>
         </is>
       </c>
       <c r="F10" t="b">
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>78.68485143096366</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>99.99996360706962</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
         <v>4</v>
@@ -6515,17 +6515,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.0126</t>
+          <t>1.0792</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.711</t>
+          <t>0.756</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.443</t>
+          <t>1.540</t>
         </is>
       </c>
       <c r="F11" t="b">
@@ -6535,7 +6535,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>99.99982965062681</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
         <v>4</v>
@@ -6556,17 +6556,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.2047</t>
+          <t>1.2431</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.705</t>
+          <t>0.726</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2.059</t>
+          <t>2.128</t>
         </is>
       </c>
       <c r="F12" t="b">
@@ -6576,7 +6576,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>99.99801771045323</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -6597,17 +6597,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.3096</t>
+          <t>0.3143</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.098</t>
+          <t>0.100</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>0.974</t>
+          <t>0.989</t>
         </is>
       </c>
       <c r="F13" t="b">
@@ -6617,7 +6617,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>99.99881055196656</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
         <v>4</v>
@@ -6918,27 +6918,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.1300</t>
+          <t>1.2703</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1.042</t>
+          <t>1.161</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.226</t>
+          <t>1.389</t>
         </is>
       </c>
       <c r="F22" t="b">
         <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>38.52515852264099</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>99.99996360706962</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
         <v>4</v>
@@ -6959,17 +6959,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.0514</t>
+          <t>1.1205</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.912</t>
+          <t>0.968</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.212</t>
+          <t>1.297</t>
         </is>
       </c>
       <c r="F23" t="b">
@@ -6979,7 +6979,7 @@
         <v>0.0002633315537803882</v>
       </c>
       <c r="H23" t="n">
-        <v>99.99982965062681</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
         <v>4</v>
@@ -7000,17 +7000,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1.9069</t>
+          <t>1.9621</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1.551</t>
+          <t>1.591</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2.345</t>
+          <t>2.420</t>
         </is>
       </c>
       <c r="F24" t="b">
@@ -7020,7 +7020,7 @@
         <v>0.002196355696408192</v>
       </c>
       <c r="H24" t="n">
-        <v>99.99801771045323</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
         <v>4</v>
@@ -7041,17 +7041,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1.3416</t>
+          <t>1.3618</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>1.021</t>
+          <t>1.034</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.763</t>
+          <t>1.793</t>
         </is>
       </c>
       <c r="F25" t="b">
@@ -7061,7 +7061,7 @@
         <v>0.002465793332856014</v>
       </c>
       <c r="H25" t="n">
-        <v>99.99881055196656</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
         <v>4</v>
@@ -7362,17 +7362,17 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>1.3039</t>
+          <t>1.5192</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>1.198</t>
+          <t>1.387</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.419</t>
+          <t>1.663</t>
         </is>
       </c>
       <c r="F34" t="b">
@@ -7382,7 +7382,7 @@
         <v>1.592719558542871e-06</v>
       </c>
       <c r="H34" t="n">
-        <v>99.99996360706962</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
         <v>4</v>
@@ -7403,17 +7403,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1.2031</t>
+          <t>1.2822</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1.031</t>
+          <t>1.095</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.404</t>
+          <t>1.502</t>
         </is>
       </c>
       <c r="F35" t="b">
@@ -7423,7 +7423,7 @@
         <v>0.00158215660418437</v>
       </c>
       <c r="H35" t="n">
-        <v>99.99982965062681</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>4</v>
@@ -7444,7 +7444,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1.2565</t>
+          <t>1.2647</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -7454,17 +7454,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.609</t>
+          <t>1.631</t>
         </is>
       </c>
       <c r="F36" t="b">
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>99.99998493565828</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>99.99801771045323</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
         <v>4</v>
@@ -7485,17 +7485,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>1.1224</t>
+          <t>1.1393</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>0.730</t>
+          <t>0.740</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>1.725</t>
+          <t>1.754</t>
         </is>
       </c>
       <c r="F37" t="b">
@@ -7505,7 +7505,7 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>99.99881055196656</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
         <v>4</v>
@@ -7806,17 +7806,17 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>1.1539</t>
+          <t>1.1959</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>1.050</t>
+          <t>1.086</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.268</t>
+          <t>1.317</t>
         </is>
       </c>
       <c r="F46" t="b">
@@ -7826,7 +7826,7 @@
         <v>1.592719558542871e-06</v>
       </c>
       <c r="H46" t="n">
-        <v>38.52515852264099</v>
+        <v>0</v>
       </c>
       <c r="I46" t="n">
         <v>4</v>
@@ -7888,24 +7888,24 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>0.6589</t>
+          <t>0.6445</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>0.507</t>
+          <t>0.494</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>0.857</t>
+          <t>0.842</t>
         </is>
       </c>
       <c r="F48" t="b">
         <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>99.99998493565828</v>
+        <v>0</v>
       </c>
       <c r="H48" t="n">
         <v>0.002196355696408192</v>
@@ -8381,17 +8381,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3.0102</t>
+          <t>3.1946</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2.119</t>
+          <t>2.246</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>4.276</t>
+          <t>4.544</t>
         </is>
       </c>
       <c r="F11" t="b">
@@ -8401,7 +8401,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>99.99999803708718</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
         <v>22</v>
@@ -8463,17 +8463,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.0133</t>
+          <t>1.0288</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.373</t>
+          <t>0.379</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>2.751</t>
+          <t>2.794</t>
         </is>
       </c>
       <c r="F13" t="b">
@@ -8483,7 +8483,7 @@
         <v>0</v>
       </c>
       <c r="H13" t="n">
-        <v>99.99372184353503</v>
+        <v>0</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -8825,27 +8825,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.0247</t>
+          <t>1.0552</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.889</t>
+          <t>0.909</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.181</t>
+          <t>1.225</t>
         </is>
       </c>
       <c r="F23" t="b">
         <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>89.05825463352933</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>99.99999803708718</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
         <v>22</v>
@@ -8866,24 +8866,24 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.7682</t>
+          <t>0.7525</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.625</t>
+          <t>0.611</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0.944</t>
+          <t>0.927</t>
         </is>
       </c>
       <c r="F24" t="b">
         <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>99.97344800904655</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
         <v>0.00288422364583929</v>
@@ -8907,7 +8907,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>1.2180</t>
+          <t>1.2225</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -8917,17 +8917,17 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.627</t>
+          <t>1.639</t>
         </is>
       </c>
       <c r="F25" t="b">
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>99.96015548986463</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
-        <v>99.99372184353503</v>
+        <v>0</v>
       </c>
       <c r="I25" t="n">
         <v>22</v>
@@ -9269,17 +9269,17 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1.1830</t>
+          <t>1.2554</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1.025</t>
+          <t>1.084</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.365</t>
+          <t>1.454</t>
         </is>
       </c>
       <c r="F35" t="b">
@@ -9289,7 +9289,7 @@
         <v>62.15076815742187</v>
       </c>
       <c r="H35" t="n">
-        <v>99.99999803708718</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>22</v>
@@ -9310,24 +9310,24 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1.1584</t>
+          <t>1.1309</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>0.929</t>
+          <t>0.904</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>1.444</t>
+          <t>1.415</t>
         </is>
       </c>
       <c r="F36" t="b">
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>99.99503978336416</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
         <v>0.00288422364583929</v>
@@ -9339,7 +9339,7 @@
         <v>22</v>
       </c>
       <c r="K36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -9351,17 +9351,17 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>1.6516</t>
+          <t>1.6744</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>1.098</t>
+          <t>1.112</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>2.484</t>
+          <t>2.522</t>
         </is>
       </c>
       <c r="F37" t="b">
@@ -9371,7 +9371,7 @@
         <v>0</v>
       </c>
       <c r="H37" t="n">
-        <v>99.99372184353503</v>
+        <v>0</v>
       </c>
       <c r="I37" t="n">
         <v>22</v>
@@ -9713,17 +9713,17 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>1.1545</t>
+          <t>1.1897</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>0.980</t>
+          <t>1.006</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1.361</t>
+          <t>1.406</t>
         </is>
       </c>
       <c r="F47" t="b">
@@ -9733,7 +9733,7 @@
         <v>62.15076815742187</v>
       </c>
       <c r="H47" t="n">
-        <v>89.05825463352933</v>
+        <v>0</v>
       </c>
       <c r="I47" t="n">
         <v>22</v>
@@ -9754,27 +9754,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>1.5080</t>
+          <t>1.5029</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>1.190</t>
+          <t>1.178</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1.912</t>
+          <t>1.917</t>
         </is>
       </c>
       <c r="F48" t="b">
         <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>99.99503978336416</v>
+        <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>99.97344800904655</v>
+        <v>0</v>
       </c>
       <c r="I48" t="n">
         <v>22</v>
@@ -9795,17 +9795,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1.3560</t>
+          <t>1.3696</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>0.891</t>
+          <t>0.899</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2.064</t>
+          <t>2.087</t>
         </is>
       </c>
       <c r="F49" t="b">
@@ -9815,7 +9815,7 @@
         <v>0</v>
       </c>
       <c r="H49" t="n">
-        <v>99.96015548986463</v>
+        <v>0</v>
       </c>
       <c r="I49" t="n">
         <v>22</v>
@@ -10206,27 +10206,27 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>0.8123</t>
+          <t>0.7257</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.648</t>
+          <t>0.533</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.018</t>
+          <t>0.988</t>
         </is>
       </c>
       <c r="F10" t="b">
         <v>1</v>
       </c>
       <c r="G10" t="n">
-        <v>99.99999999000001</v>
+        <v>0</v>
       </c>
       <c r="H10" t="n">
-        <v>99.99999971390291</v>
+        <v>0</v>
       </c>
       <c r="I10" t="n">
         <v>22</v>
@@ -10247,17 +10247,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.3476</t>
+          <t>1.4276</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.945</t>
+          <t>0.999</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.923</t>
+          <t>2.040</t>
         </is>
       </c>
       <c r="F11" t="b">
@@ -10267,7 +10267,7 @@
         <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>99.99994153729666</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
         <v>22</v>
@@ -10288,17 +10288,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>0.8599</t>
+          <t>0.8876</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.425</t>
+          <t>0.438</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.741</t>
+          <t>1.799</t>
         </is>
       </c>
       <c r="F12" t="b">
@@ -10308,7 +10308,7 @@
         <v>0</v>
       </c>
       <c r="H12" t="n">
-        <v>99.99999916573678</v>
+        <v>0</v>
       </c>
       <c r="I12" t="n">
         <v>0</v>
@@ -10650,27 +10650,27 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.9105</t>
+          <t>0.9543</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.837</t>
+          <t>0.866</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0.991</t>
+          <t>1.051</t>
         </is>
       </c>
       <c r="F22" t="b">
         <v>1</v>
       </c>
       <c r="G22" t="n">
-        <v>99.99999341688996</v>
+        <v>0</v>
       </c>
       <c r="H22" t="n">
-        <v>99.99999971390291</v>
+        <v>0</v>
       </c>
       <c r="I22" t="n">
         <v>22</v>
@@ -10691,27 +10691,27 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.2654</t>
+          <t>1.2930</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.098</t>
+          <t>1.113</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.458</t>
+          <t>1.501</t>
         </is>
       </c>
       <c r="F23" t="b">
         <v>1</v>
       </c>
       <c r="G23" t="n">
-        <v>99.996277246481</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>99.99994153729666</v>
+        <v>0</v>
       </c>
       <c r="I23" t="n">
         <v>22</v>
@@ -10732,27 +10732,27 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1.1252</t>
+          <t>1.1370</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.901</t>
+          <t>0.905</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.406</t>
+          <t>1.429</t>
         </is>
       </c>
       <c r="F24" t="b">
         <v>1</v>
       </c>
       <c r="G24" t="n">
-        <v>99.99525725585139</v>
+        <v>0</v>
       </c>
       <c r="H24" t="n">
-        <v>99.99999916573678</v>
+        <v>0</v>
       </c>
       <c r="I24" t="n">
         <v>22</v>
@@ -10773,24 +10773,24 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.5440</t>
+          <t>0.5389</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.399</t>
+          <t>0.394</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0.742</t>
+          <t>0.737</t>
         </is>
       </c>
       <c r="F25" t="b">
         <v>1</v>
       </c>
       <c r="G25" t="n">
-        <v>99.99923978474666</v>
+        <v>0</v>
       </c>
       <c r="H25" t="n">
         <v>0.0007096613591267564</v>
@@ -11094,27 +11094,27 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>0.9743</t>
+          <t>1.1041</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>0.898</t>
+          <t>1.010</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>1.057</t>
+          <t>1.206</t>
         </is>
       </c>
       <c r="F34" t="b">
         <v>1</v>
       </c>
       <c r="G34" t="n">
-        <v>19.81185314384397</v>
+        <v>0</v>
       </c>
       <c r="H34" t="n">
-        <v>99.99999971390291</v>
+        <v>0</v>
       </c>
       <c r="I34" t="n">
         <v>22</v>
@@ -11135,27 +11135,27 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>1.3261</t>
+          <t>1.3606</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>1.143</t>
+          <t>1.164</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>1.539</t>
+          <t>1.591</t>
         </is>
       </c>
       <c r="F35" t="b">
         <v>1</v>
       </c>
       <c r="G35" t="n">
-        <v>99.98669975490962</v>
+        <v>0</v>
       </c>
       <c r="H35" t="n">
-        <v>99.99994153729666</v>
+        <v>0</v>
       </c>
       <c r="I35" t="n">
         <v>22</v>
@@ -11176,7 +11176,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>1.6560</t>
+          <t>1.6672</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -11186,17 +11186,17 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>2.088</t>
+          <t>2.116</t>
         </is>
       </c>
       <c r="F36" t="b">
         <v>1</v>
       </c>
       <c r="G36" t="n">
-        <v>99.99979978102513</v>
+        <v>0</v>
       </c>
       <c r="H36" t="n">
-        <v>99.99999916573678</v>
+        <v>0</v>
       </c>
       <c r="I36" t="n">
         <v>22</v>
@@ -11538,27 +11538,27 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>1.0700</t>
+          <t>1.1569</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>0.977</t>
+          <t>1.049</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>1.172</t>
+          <t>1.276</t>
         </is>
       </c>
       <c r="F46" t="b">
         <v>1</v>
       </c>
       <c r="G46" t="n">
-        <v>19.81185314384397</v>
+        <v>0</v>
       </c>
       <c r="H46" t="n">
-        <v>99.99999341688996</v>
+        <v>0</v>
       </c>
       <c r="I46" t="n">
         <v>22</v>
@@ -11579,27 +11579,27 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>1.0480</t>
+          <t>1.0523</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>0.887</t>
+          <t>0.884</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>1.239</t>
+          <t>1.252</t>
         </is>
       </c>
       <c r="F47" t="b">
         <v>1</v>
       </c>
       <c r="G47" t="n">
-        <v>99.98669975490962</v>
+        <v>0</v>
       </c>
       <c r="H47" t="n">
-        <v>99.996277246481</v>
+        <v>0</v>
       </c>
       <c r="I47" t="n">
         <v>22</v>
@@ -11620,27 +11620,27 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>1.4717</t>
+          <t>1.4663</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>1.135</t>
+          <t>1.124</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>1.909</t>
+          <t>1.913</t>
         </is>
       </c>
       <c r="F48" t="b">
         <v>1</v>
       </c>
       <c r="G48" t="n">
-        <v>99.99979978102513</v>
+        <v>0</v>
       </c>
       <c r="H48" t="n">
-        <v>99.99525725585139</v>
+        <v>0</v>
       </c>
       <c r="I48" t="n">
         <v>22</v>
@@ -11661,17 +11661,17 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>1.5183</t>
+          <t>1.5326</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>1.007</t>
+          <t>1.015</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>2.289</t>
+          <t>2.314</t>
         </is>
       </c>
       <c r="F49" t="b">
@@ -11681,7 +11681,7 @@
         <v>0</v>
       </c>
       <c r="H49" t="n">
-        <v>99.99923978474666</v>
+        <v>0</v>
       </c>
       <c r="I49" t="n">
         <v>22</v>
@@ -11982,17 +11982,17 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>2.4413</t>
+          <t>2.8088</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>2.019</t>
+          <t>2.316</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>2.952</t>
+          <t>3.406</t>
         </is>
       </c>
       <c r="F58" t="b">
@@ -12002,7 +12002,7 @@
         <v>0.0004117208146238172</v>
       </c>
       <c r="H58" t="n">
-        <v>99.99999971390291</v>
+        <v>0</v>
       </c>
       <c r="I58" t="n">
         <v>22</v>
@@ -12011,7 +12011,7 @@
         <v>22</v>
       </c>
       <c r="K58" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="59">
@@ -12023,27 +12023,27 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>0.7422</t>
+          <t>0.7242</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>0.539</t>
+          <t>0.506</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>1.023</t>
+          <t>1.036</t>
         </is>
       </c>
       <c r="F59" t="b">
         <v>1</v>
       </c>
       <c r="G59" t="n">
-        <v>99.99999999000001</v>
+        <v>0</v>
       </c>
       <c r="H59" t="n">
-        <v>99.99994153729666</v>
+        <v>0</v>
       </c>
       <c r="I59" t="n">
         <v>22</v>
@@ -12064,17 +12064,17 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>1.1505</t>
+          <t>1.1835</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>0.561</t>
+          <t>0.576</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>2.361</t>
+          <t>2.431</t>
         </is>
       </c>
       <c r="F60" t="b">
@@ -12084,7 +12084,7 @@
         <v>0</v>
       </c>
       <c r="H60" t="n">
-        <v>99.99999916573678</v>
+        <v>0</v>
       </c>
       <c r="I60" t="n">
         <v>22</v>
@@ -12426,17 +12426,17 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>2.6812</t>
+          <t>2.9432</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>2.208</t>
+          <t>2.417</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>3.256</t>
+          <t>3.585</t>
         </is>
       </c>
       <c r="F70" t="b">
@@ -12446,7 +12446,7 @@
         <v>0.0004117208146238172</v>
       </c>
       <c r="H70" t="n">
-        <v>99.99999341688996</v>
+        <v>0</v>
       </c>
       <c r="I70" t="n">
         <v>22</v>
@@ -12467,27 +12467,27 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>0.5866</t>
+          <t>0.5601</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>0.422</t>
+          <t>0.389</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>0.816</t>
+          <t>0.807</t>
         </is>
       </c>
       <c r="F71" t="b">
         <v>1</v>
       </c>
       <c r="G71" t="n">
-        <v>99.99999999000001</v>
+        <v>0</v>
       </c>
       <c r="H71" t="n">
-        <v>99.996277246481</v>
+        <v>0</v>
       </c>
       <c r="I71" t="n">
         <v>22</v>
@@ -12508,17 +12508,17 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>1.0225</t>
+          <t>1.0409</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>0.493</t>
+          <t>0.502</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>2.119</t>
+          <t>2.159</t>
         </is>
       </c>
       <c r="F72" t="b">
@@ -12528,7 +12528,7 @@
         <v>0</v>
       </c>
       <c r="H72" t="n">
-        <v>99.99525725585139</v>
+        <v>0</v>
       </c>
       <c r="I72" t="n">
         <v>22</v>
@@ -12549,17 +12549,17 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>5.3330</t>
+          <t>5.3897</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>1.946</t>
+          <t>1.965</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>14.616</t>
+          <t>14.781</t>
         </is>
       </c>
       <c r="F73" t="b">
@@ -12569,7 +12569,7 @@
         <v>0</v>
       </c>
       <c r="H73" t="n">
-        <v>99.99923978474666</v>
+        <v>0</v>
       </c>
       <c r="I73" t="n">
         <v>0</v>
@@ -12870,17 +12870,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>2.5057</t>
+          <t>2.5441</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>2.066</t>
+          <t>2.097</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>3.039</t>
+          <t>3.087</t>
         </is>
       </c>
       <c r="F82" t="b">
@@ -12890,7 +12890,7 @@
         <v>0.0004117208146238172</v>
       </c>
       <c r="H82" t="n">
-        <v>19.81185314384397</v>
+        <v>0</v>
       </c>
       <c r="I82" t="n">
         <v>22</v>
@@ -12911,27 +12911,27 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>0.5597</t>
+          <t>0.5323</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>0.401</t>
+          <t>0.368</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>0.781</t>
+          <t>0.770</t>
         </is>
       </c>
       <c r="F83" t="b">
         <v>1</v>
       </c>
       <c r="G83" t="n">
-        <v>99.99999999000001</v>
+        <v>0</v>
       </c>
       <c r="H83" t="n">
-        <v>99.98669975490962</v>
+        <v>0</v>
       </c>
       <c r="I83" t="n">
         <v>22</v>
@@ -12952,17 +12952,17 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>0.6948</t>
+          <t>0.7099</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>0.334</t>
+          <t>0.341</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>1.444</t>
+          <t>1.477</t>
         </is>
       </c>
       <c r="F84" t="b">
@@ -12972,7 +12972,7 @@
         <v>0</v>
       </c>
       <c r="H84" t="n">
-        <v>99.99979978102513</v>
+        <v>0</v>
       </c>
       <c r="I84" t="n">
         <v>22</v>
@@ -13072,7 +13072,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>DELTA_INAPPLICABLE</t>
+          <t>INSUFFICIENT_SIGNAL</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -13184,10 +13184,10 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E5" t="n">
         <v>2</v>
@@ -13238,10 +13238,10 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E7" t="n">
         <v>5</v>
@@ -13265,10 +13265,10 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D8" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="E8" t="n">
         <v>4</v>
@@ -14927,38 +14927,36 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L20" t="n">
-        <v>99.99836701224508</v>
+        <v>99.89803107234498</v>
       </c>
       <c r="M20" t="n">
-        <v>99.99836701224508</v>
+        <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>99.99836701224508</v>
+        <v>0</v>
       </c>
       <c r="O20" t="n">
-        <v>99.99836701224508</v>
+        <v>0</v>
       </c>
       <c r="P20" t="n">
         <v>1.857918797720702e-05</v>
       </c>
-      <c r="Q20" t="n">
-        <v>0.2447791366789677</v>
-      </c>
+      <c r="Q20" t="inlineStr"/>
       <c r="R20" t="n">
-        <v>0.00163346758135682</v>
+        <v>0.001467078559092024</v>
       </c>
       <c r="S20" t="n">
-        <v>0.001114210250503705</v>
+        <v>0.0009750436212635123</v>
       </c>
       <c r="T20" t="n">
-        <v>0.0001056016389969581</v>
+        <v>2.624452291287189e-05</v>
       </c>
       <c r="U20" t="n">
-        <v>0.001080148172350531</v>
+        <v>0.0009458711353828253</v>
       </c>
       <c r="V20" t="n">
         <v>45</v>
@@ -15009,11 +15007,11 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L21" t="n">
-        <v>99.98082748850817</v>
+        <v>0.0005314895659107588</v>
       </c>
       <c r="M21" t="n">
         <v>0</v>
@@ -15027,9 +15025,7 @@
       <c r="P21" t="n">
         <v>1.866051916918061e-05</v>
       </c>
-      <c r="Q21" t="n">
-        <v>13927914.16784326</v>
-      </c>
+      <c r="Q21" t="inlineStr"/>
       <c r="R21" t="n">
         <v>0.001598895696833926</v>
       </c>
@@ -15091,38 +15087,36 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L22" t="n">
-        <v>67.15278858582882</v>
+        <v>99.99604338082898</v>
       </c>
       <c r="M22" t="n">
-        <v>67.15278858582882</v>
+        <v>0</v>
       </c>
       <c r="N22" t="n">
-        <v>67.15278858582882</v>
+        <v>0</v>
       </c>
       <c r="O22" t="n">
-        <v>67.15278858582882</v>
+        <v>0</v>
       </c>
       <c r="P22" t="n">
         <v>2.670577428594451e-05</v>
       </c>
-      <c r="Q22" t="n">
-        <v>14766364.29839349</v>
-      </c>
+      <c r="Q22" t="inlineStr"/>
       <c r="R22" t="n">
-        <v>0.001722193049745661</v>
+        <v>0.001591851093980468</v>
       </c>
       <c r="S22" t="n">
-        <v>0.001189969912825443</v>
+        <v>0.001076721425630619</v>
       </c>
       <c r="T22" t="n">
-        <v>0.0002275462145916859</v>
+        <v>0.0001741717392829618</v>
       </c>
       <c r="U22" t="n">
-        <v>0.001149665262185615</v>
+        <v>0.001041921884216244</v>
       </c>
       <c r="V22" t="n">
         <v>45</v>
@@ -17451,38 +17445,36 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L51" t="n">
-        <v>20.17276949813065</v>
+        <v>0.002450913499673524</v>
       </c>
       <c r="M51" t="n">
-        <v>20.17276949813065</v>
+        <v>0</v>
       </c>
       <c r="N51" t="n">
-        <v>20.17276949813065</v>
+        <v>0</v>
       </c>
       <c r="O51" t="n">
-        <v>20.17276949813065</v>
+        <v>0</v>
       </c>
       <c r="P51" t="n">
         <v>1.712831358017336e-05</v>
       </c>
-      <c r="Q51" t="n">
-        <v>8947471.209929135</v>
-      </c>
+      <c r="Q51" t="inlineStr"/>
       <c r="R51" t="n">
-        <v>0.001695889896326707</v>
+        <v>0.001653828431228948</v>
       </c>
       <c r="S51" t="n">
-        <v>0.001215350627910184</v>
+        <v>0.001180192856083302</v>
       </c>
       <c r="T51" t="n">
-        <v>6.822928405279572e-05</v>
+        <v>8.000746761023135e-05</v>
       </c>
       <c r="U51" t="n">
-        <v>0.001199116567817804</v>
+        <v>0.001164314193467678</v>
       </c>
       <c r="V51" t="n">
         <v>45</v>
@@ -17773,7 +17765,7 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L55" t="n">
@@ -18335,38 +18327,36 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L62" t="n">
-        <v>0.4381125719082086</v>
+        <v>1.278761050355924e-10</v>
       </c>
       <c r="M62" t="n">
-        <v>0.4381125719082086</v>
+        <v>0</v>
       </c>
       <c r="N62" t="n">
-        <v>0.4381125719082086</v>
+        <v>0</v>
       </c>
       <c r="O62" t="n">
-        <v>0.4381125719082086</v>
+        <v>0</v>
       </c>
       <c r="P62" t="n">
         <v>0.006028409511812455</v>
       </c>
-      <c r="Q62" t="n">
-        <v>0.190690661639951</v>
-      </c>
+      <c r="Q62" t="inlineStr"/>
       <c r="R62" t="n">
-        <v>0.7057971357643902</v>
+        <v>0.5872347740240069</v>
       </c>
       <c r="S62" t="n">
-        <v>0.4542934887457543</v>
+        <v>0.3670636316124459</v>
       </c>
       <c r="T62" t="n">
-        <v>0.02161838133580918</v>
+        <v>0.04441756303840405</v>
       </c>
       <c r="U62" t="n">
-        <v>0.4755439613080352</v>
+        <v>0.3836213737902346</v>
       </c>
       <c r="V62" t="n">
         <v>41</v>
@@ -18417,38 +18407,36 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L63" t="n">
-        <v>0.368184590370468</v>
+        <v>8.945047182007545e-15</v>
       </c>
       <c r="M63" t="n">
-        <v>0.368184590370468</v>
+        <v>0</v>
       </c>
       <c r="N63" t="n">
-        <v>0.368184590370468</v>
+        <v>0</v>
       </c>
       <c r="O63" t="n">
-        <v>0.368184590370468</v>
+        <v>0</v>
       </c>
       <c r="P63" t="n">
         <v>0.006041416232669848</v>
       </c>
-      <c r="Q63" t="n">
-        <v>1281490779.838289</v>
-      </c>
+      <c r="Q63" t="inlineStr"/>
       <c r="R63" t="n">
-        <v>0.5480529557596417</v>
+        <v>0.4830169501854772</v>
       </c>
       <c r="S63" t="n">
-        <v>0.3537164742715944</v>
+        <v>0.3035211287507119</v>
       </c>
       <c r="T63" t="n">
-        <v>0.05194639051618588</v>
+        <v>0.01522610864425911</v>
       </c>
       <c r="U63" t="n">
-        <v>0.3698125409926292</v>
+        <v>0.3176971655586485</v>
       </c>
       <c r="V63" t="n">
         <v>41</v>
@@ -19811,38 +19799,36 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L80" t="n">
-        <v>99.99999874596539</v>
+        <v>99.99315761885542</v>
       </c>
       <c r="M80" t="n">
-        <v>99.99999874596539</v>
+        <v>0</v>
       </c>
       <c r="N80" t="n">
-        <v>99.99999874596539</v>
+        <v>0</v>
       </c>
       <c r="O80" t="n">
-        <v>99.99999874596539</v>
+        <v>0</v>
       </c>
       <c r="P80" t="n">
         <v>2.410448287007926e-05</v>
       </c>
-      <c r="Q80" t="n">
-        <v>0.273595803050369</v>
-      </c>
+      <c r="Q80" t="inlineStr"/>
       <c r="R80" t="n">
-        <v>0.001938011527537108</v>
+        <v>0.001716144095571411</v>
       </c>
       <c r="S80" t="n">
-        <v>0.00124428403281424</v>
+        <v>0.001075797348003461</v>
       </c>
       <c r="T80" t="n">
-        <v>8.490851128771211e-05</v>
+        <v>2.646742971968569e-05</v>
       </c>
       <c r="U80" t="n">
-        <v>0.00130236131674547</v>
+        <v>0.001126349212955512</v>
       </c>
       <c r="V80" t="n">
         <v>41</v>
@@ -19893,38 +19879,36 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L81" t="n">
-        <v>0.004735882525673585</v>
+        <v>99.9998928058157</v>
       </c>
       <c r="M81" t="n">
-        <v>0.004735882525673585</v>
+        <v>0</v>
       </c>
       <c r="N81" t="n">
-        <v>0.004735882525673585</v>
+        <v>0</v>
       </c>
       <c r="O81" t="n">
-        <v>0.004735882525673585</v>
+        <v>0</v>
       </c>
       <c r="P81" t="n">
         <v>1.006199791036633e-05</v>
       </c>
-      <c r="Q81" t="n">
-        <v>1592103.743332472</v>
-      </c>
+      <c r="Q81" t="inlineStr"/>
       <c r="R81" t="n">
-        <v>0.0007968359450181702</v>
+        <v>0.0007968338020428505</v>
       </c>
       <c r="S81" t="n">
-        <v>0.0005261200987242614</v>
+        <v>0.0005261183540943751</v>
       </c>
       <c r="T81" t="n">
-        <v>9.882015128152496e-05</v>
+        <v>9.881858132556286e-05</v>
       </c>
       <c r="U81" t="n">
-        <v>0.0005491555906107161</v>
+        <v>0.0005491538105611956</v>
       </c>
       <c r="V81" t="n">
         <v>41</v>
@@ -20057,38 +20041,36 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L83" t="n">
-        <v>99.98397501305337</v>
+        <v>98.75610295753103</v>
       </c>
       <c r="M83" t="n">
-        <v>99.98397501305337</v>
+        <v>0</v>
       </c>
       <c r="N83" t="n">
-        <v>99.98397501305337</v>
+        <v>0</v>
       </c>
       <c r="O83" t="n">
-        <v>99.98397501305337</v>
+        <v>0</v>
       </c>
       <c r="P83" t="n">
         <v>8.630764042192715e-06</v>
       </c>
-      <c r="Q83" t="n">
-        <v>0.5416440336051862</v>
-      </c>
+      <c r="Q83" t="inlineStr"/>
       <c r="R83" t="n">
-        <v>0.0007645859154417622</v>
+        <v>0.0007263137477559209</v>
       </c>
       <c r="S83" t="n">
-        <v>0.0004942381645320634</v>
+        <v>0.0004649630714829625</v>
       </c>
       <c r="T83" t="n">
-        <v>4.430887812567272e-05</v>
+        <v>3.176907030865317e-05</v>
       </c>
       <c r="U83" t="n">
-        <v>0.0005172417758557939</v>
+        <v>0.0004866826278176599</v>
       </c>
       <c r="V83" t="n">
         <v>41</v>
@@ -20385,11 +20367,11 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L87" t="n">
-        <v>99.98869119254518</v>
+        <v>99.3020403130092</v>
       </c>
       <c r="M87" t="n">
         <v>0</v>
@@ -20403,9 +20385,7 @@
       <c r="P87" t="n">
         <v>6.485511828967794e-06</v>
       </c>
-      <c r="Q87" t="n">
-        <v>6255021.703480332</v>
-      </c>
+      <c r="Q87" t="inlineStr"/>
       <c r="R87" t="n">
         <v>0.0005515883915342586</v>
       </c>
@@ -20467,11 +20447,11 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L88" t="n">
-        <v>99.9989016016915</v>
+        <v>5.711663740193273e-05</v>
       </c>
       <c r="M88" t="n">
         <v>0</v>
@@ -20485,9 +20465,7 @@
       <c r="P88" t="n">
         <v>2.451821705490913e-05</v>
       </c>
-      <c r="Q88" t="n">
-        <v>19408134.82491929</v>
-      </c>
+      <c r="Q88" t="inlineStr"/>
       <c r="R88" t="n">
         <v>0.002237294645361168</v>
       </c>
@@ -20795,38 +20773,36 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L92" t="n">
-        <v>0.4537941446299353</v>
+        <v>3.23273682366202e-12</v>
       </c>
       <c r="M92" t="n">
-        <v>0.4537941446299353</v>
+        <v>0</v>
       </c>
       <c r="N92" t="n">
-        <v>0.4537941446299353</v>
+        <v>0</v>
       </c>
       <c r="O92" t="n">
-        <v>0.4537941446299353</v>
+        <v>0</v>
       </c>
       <c r="P92" t="n">
         <v>0.006013021016645737</v>
       </c>
-      <c r="Q92" t="n">
-        <v>0.2053037849078561</v>
-      </c>
+      <c r="Q92" t="inlineStr"/>
       <c r="R92" t="n">
-        <v>0.7840396962739421</v>
+        <v>0.6513349590144611</v>
       </c>
       <c r="S92" t="n">
-        <v>0.3810602543943351</v>
+        <v>0.3051981445436431</v>
       </c>
       <c r="T92" t="n">
-        <v>0.02318843586393549</v>
+        <v>0.04283588671188832</v>
       </c>
       <c r="U92" t="n">
-        <v>0.4761401898876165</v>
+        <v>0.3802972005941919</v>
       </c>
       <c r="V92" t="n">
         <v>35</v>
@@ -21369,38 +21345,36 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L99" t="n">
-        <v>5.144869335656168</v>
+        <v>7.100089660627878</v>
       </c>
       <c r="M99" t="n">
-        <v>5.144869335656168</v>
+        <v>0</v>
       </c>
       <c r="N99" t="n">
-        <v>5.144869335656168</v>
+        <v>0</v>
       </c>
       <c r="O99" t="n">
-        <v>5.144869335656168</v>
+        <v>0</v>
       </c>
       <c r="P99" t="n">
         <v>0.001212733279543603</v>
       </c>
-      <c r="Q99" t="n">
-        <v>0.2926929975019416</v>
-      </c>
+      <c r="Q99" t="inlineStr"/>
       <c r="R99" t="n">
-        <v>0.1078019264456274</v>
+        <v>0.08222782261162327</v>
       </c>
       <c r="S99" t="n">
-        <v>0.05457194168178857</v>
+        <v>0.03897772604259196</v>
       </c>
       <c r="T99" t="n">
-        <v>0.009002522277096664</v>
+        <v>0.001463525737282649</v>
       </c>
       <c r="U99" t="n">
-        <v>0.06804964171747295</v>
+        <v>0.04870882681814144</v>
       </c>
       <c r="V99" t="n">
         <v>35</v>
@@ -21615,38 +21589,36 @@
       </c>
       <c r="K102" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L102" t="n">
-        <v>12.94399970085989</v>
+        <v>3.876759057336397e-07</v>
       </c>
       <c r="M102" t="n">
-        <v>12.94399970085989</v>
+        <v>0</v>
       </c>
       <c r="N102" t="n">
-        <v>12.94399970085989</v>
+        <v>0</v>
       </c>
       <c r="O102" t="n">
-        <v>12.94399970085989</v>
+        <v>0</v>
       </c>
       <c r="P102" t="n">
         <v>0.0004781921699441366</v>
       </c>
-      <c r="Q102" t="n">
-        <v>0.276495883647545</v>
-      </c>
+      <c r="Q102" t="inlineStr"/>
       <c r="R102" t="n">
-        <v>0.04199901033481993</v>
+        <v>0.0321830166491119</v>
       </c>
       <c r="S102" t="n">
-        <v>0.02117740292989744</v>
+        <v>0.01522063651010338</v>
       </c>
       <c r="T102" t="n">
-        <v>0.002978172244975777</v>
+        <v>0.0007795757489196533</v>
       </c>
       <c r="U102" t="n">
-        <v>0.02641940342858014</v>
+        <v>0.01901992103434821</v>
       </c>
       <c r="V102" t="n">
         <v>35</v>
@@ -22271,20 +22243,20 @@
       </c>
       <c r="K110" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L110" t="n">
         <v>99.99832749090832</v>
       </c>
       <c r="M110" t="n">
-        <v>99.99832749090832</v>
+        <v>0</v>
       </c>
       <c r="N110" t="n">
-        <v>99.99832749090832</v>
+        <v>0</v>
       </c>
       <c r="O110" t="n">
-        <v>99.99832749090832</v>
+        <v>0</v>
       </c>
       <c r="P110" t="n">
         <v>2.483947791541276e-05</v>
@@ -22293,16 +22265,16 @@
         <v>0.234306827612376</v>
       </c>
       <c r="R110" t="n">
-        <v>0.002357012541565787</v>
+        <v>0.002070181323649837</v>
       </c>
       <c r="S110" t="n">
-        <v>0.001165694379217539</v>
+        <v>0.0009921092319155555</v>
       </c>
       <c r="T110" t="n">
-        <v>0.0001028130738700687</v>
+        <v>3.831768508750621e-05</v>
       </c>
       <c r="U110" t="n">
-        <v>0.001456206792707133</v>
+        <v>0.001239998601838677</v>
       </c>
       <c r="V110" t="n">
         <v>35</v>
@@ -22353,38 +22325,36 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L111" t="n">
-        <v>18.07141117982593</v>
+        <v>1</v>
       </c>
       <c r="M111" t="n">
-        <v>18.07141117982593</v>
+        <v>0</v>
       </c>
       <c r="N111" t="n">
-        <v>18.07141117982593</v>
+        <v>0</v>
       </c>
       <c r="O111" t="n">
-        <v>18.07141117982593</v>
+        <v>0</v>
       </c>
       <c r="P111" t="n">
         <v>1.133492938024884e-05</v>
       </c>
-      <c r="Q111" t="n">
-        <v>3664122.387808314</v>
-      </c>
+      <c r="Q111" t="inlineStr"/>
       <c r="R111" t="n">
-        <v>0.001255930794024005</v>
+        <v>0.001238663307138183</v>
       </c>
       <c r="S111" t="n">
-        <v>0.0006177383806401349</v>
+        <v>0.0006074867904251721</v>
       </c>
       <c r="T111" t="n">
-        <v>5.185802563996097e-05</v>
+        <v>5.573383524628498e-05</v>
       </c>
       <c r="U111" t="n">
-        <v>0.0007713032139580113</v>
+        <v>0.0007584375592510155</v>
       </c>
       <c r="V111" t="n">
         <v>35</v>
@@ -22517,38 +22487,36 @@
       </c>
       <c r="K113" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L113" t="n">
-        <v>99.99655614702037</v>
+        <v>99.3020403130092</v>
       </c>
       <c r="M113" t="n">
-        <v>99.99655614702037</v>
+        <v>0</v>
       </c>
       <c r="N113" t="n">
-        <v>99.99655614702037</v>
+        <v>0</v>
       </c>
       <c r="O113" t="n">
-        <v>99.99655614702037</v>
+        <v>0</v>
       </c>
       <c r="P113" t="n">
         <v>1.159122963878005e-05</v>
       </c>
-      <c r="Q113" t="n">
-        <v>0.9187396558252575</v>
-      </c>
+      <c r="Q113" t="inlineStr"/>
       <c r="R113" t="n">
-        <v>0.0009943689457676606</v>
+        <v>0.0009380057570229976</v>
       </c>
       <c r="S113" t="n">
-        <v>0.0004907480820797233</v>
+        <v>0.0004567226564730005</v>
       </c>
       <c r="T113" t="n">
-        <v>3.074052882887063e-05</v>
+        <v>2.190425871369077e-05</v>
       </c>
       <c r="U113" t="n">
-        <v>0.0006132533836291775</v>
+        <v>0.0005707606261452159</v>
       </c>
       <c r="V113" t="n">
         <v>35</v>
@@ -22599,38 +22567,36 @@
       </c>
       <c r="K114" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L114" t="n">
-        <v>99.99883438093936</v>
+        <v>99.3020403130092</v>
       </c>
       <c r="M114" t="n">
-        <v>99.99883438093936</v>
+        <v>0</v>
       </c>
       <c r="N114" t="n">
-        <v>99.99883438093936</v>
+        <v>0</v>
       </c>
       <c r="O114" t="n">
-        <v>99.99883438093936</v>
+        <v>0</v>
       </c>
       <c r="P114" t="n">
         <v>5.189293034177101e-06</v>
       </c>
-      <c r="Q114" t="n">
-        <v>3586070.13751977</v>
-      </c>
+      <c r="Q114" t="inlineStr"/>
       <c r="R114" t="n">
-        <v>0.0005219254156982111</v>
+        <v>0.0005055773466846192</v>
       </c>
       <c r="S114" t="n">
-        <v>0.0002672525634914902</v>
+        <v>0.0002570638138923832</v>
       </c>
       <c r="T114" t="n">
-        <v>5.337654059309692e-05</v>
+        <v>4.892264629836939e-05</v>
       </c>
       <c r="U114" t="n">
-        <v>0.0003330304637794277</v>
+        <v>0.0003204102458501164</v>
       </c>
       <c r="V114" t="n">
         <v>35</v>
@@ -22681,38 +22647,36 @@
       </c>
       <c r="K115" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L115" t="n">
-        <v>73.33347320005834</v>
+        <v>99.3020403130092</v>
       </c>
       <c r="M115" t="n">
-        <v>73.33347320005834</v>
+        <v>0</v>
       </c>
       <c r="N115" t="n">
-        <v>73.33347320005834</v>
+        <v>0</v>
       </c>
       <c r="O115" t="n">
-        <v>73.33347320005834</v>
+        <v>0</v>
       </c>
       <c r="P115" t="n">
         <v>8.608843789610296e-06</v>
       </c>
-      <c r="Q115" t="n">
-        <v>3538910.768658287</v>
-      </c>
+      <c r="Q115" t="inlineStr"/>
       <c r="R115" t="n">
-        <v>0.0008725464356789725</v>
+        <v>0.0008393752056345484</v>
       </c>
       <c r="S115" t="n">
-        <v>0.0004463848235045245</v>
+        <v>0.0004256795584865307</v>
       </c>
       <c r="T115" t="n">
-        <v>6.49018135431961e-05</v>
+        <v>5.67753006828295e-05</v>
       </c>
       <c r="U115" t="n">
-        <v>0.0005569304906200015</v>
+        <v>0.000531279374617475</v>
       </c>
       <c r="V115" t="n">
         <v>35</v>
@@ -22763,38 +22727,36 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L116" t="n">
-        <v>99.88585064778931</v>
+        <v>57.24173631838615</v>
       </c>
       <c r="M116" t="n">
-        <v>99.88585064778931</v>
+        <v>0</v>
       </c>
       <c r="N116" t="n">
-        <v>99.88585064778931</v>
+        <v>0</v>
       </c>
       <c r="O116" t="n">
-        <v>99.88585064778931</v>
+        <v>0</v>
       </c>
       <c r="P116" t="n">
         <v>4.326630580658509e-06</v>
       </c>
-      <c r="Q116" t="n">
-        <v>833048.4074225093</v>
-      </c>
+      <c r="Q116" t="inlineStr"/>
       <c r="R116" t="n">
-        <v>0.000439938919140674</v>
+        <v>0.0004284616947221984</v>
       </c>
       <c r="S116" t="n">
-        <v>0.0002148986013965135</v>
+        <v>0.0002080468403985156</v>
       </c>
       <c r="T116" t="n">
-        <v>9.665022184634727e-06</v>
+        <v>1.020079760668863e-05</v>
       </c>
       <c r="U116" t="n">
-        <v>0.0002685860833727325</v>
+        <v>0.000259999796873299</v>
       </c>
       <c r="V116" t="n">
         <v>35</v>
@@ -22927,7 +22889,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L118" t="n">
@@ -22945,9 +22907,7 @@
       <c r="P118" t="n">
         <v>2.82701175668801e-05</v>
       </c>
-      <c r="Q118" t="n">
-        <v>18994601.36082338</v>
-      </c>
+      <c r="Q118" t="inlineStr"/>
       <c r="R118" t="n">
         <v>0.0007914309582418585</v>
       </c>
@@ -23337,38 +23297,36 @@
       </c>
       <c r="K123" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L123" t="n">
-        <v>0.4324265093155894</v>
+        <v>5.022565752920349e-11</v>
       </c>
       <c r="M123" t="n">
-        <v>0.4324265093155894</v>
+        <v>0</v>
       </c>
       <c r="N123" t="n">
-        <v>0.4324265093155894</v>
+        <v>0</v>
       </c>
       <c r="O123" t="n">
-        <v>0.4324265093155894</v>
+        <v>0</v>
       </c>
       <c r="P123" t="n">
         <v>0.005987173046325693</v>
       </c>
-      <c r="Q123" t="n">
-        <v>3208408205.468919</v>
-      </c>
+      <c r="Q123" t="inlineStr"/>
       <c r="R123" t="n">
-        <v>0.3741162574892581</v>
+        <v>0.3398878015445518</v>
       </c>
       <c r="S123" t="n">
-        <v>0.2082634105991247</v>
+        <v>0.1820590970145115</v>
       </c>
       <c r="T123" t="n">
-        <v>0.08975775768330374</v>
+        <v>0.05659927752523886</v>
       </c>
       <c r="U123" t="n">
-        <v>0.3245245259969843</v>
+        <v>0.2854377500649131</v>
       </c>
       <c r="V123" t="n">
         <v>34</v>
@@ -24649,38 +24607,36 @@
       </c>
       <c r="K139" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L139" t="n">
-        <v>27.49288398547458</v>
+        <v>8.531769115521261e-10</v>
       </c>
       <c r="M139" t="n">
-        <v>27.49288398547458</v>
+        <v>0</v>
       </c>
       <c r="N139" t="n">
-        <v>27.49288398547458</v>
+        <v>0</v>
       </c>
       <c r="O139" t="n">
-        <v>27.49288398547458</v>
+        <v>0</v>
       </c>
       <c r="P139" t="n">
         <v>0.0004185777354576049</v>
       </c>
-      <c r="Q139" t="n">
-        <v>70148887.23567463</v>
-      </c>
+      <c r="Q139" t="inlineStr"/>
       <c r="R139" t="n">
-        <v>0.02634880500122358</v>
+        <v>0.01878445972775438</v>
       </c>
       <c r="S139" t="n">
-        <v>0.01421937927335543</v>
+        <v>0.009126083727519309</v>
       </c>
       <c r="T139" t="n">
-        <v>0.003372141441029104</v>
+        <v>0.0008576958932341753</v>
       </c>
       <c r="U139" t="n">
-        <v>0.02235251881784544</v>
+        <v>0.01440497160124364</v>
       </c>
       <c r="V139" t="n">
         <v>34</v>
@@ -24895,38 +24851,36 @@
       </c>
       <c r="K142" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L142" t="n">
         <v>99.99996360706962</v>
       </c>
       <c r="M142" t="n">
-        <v>99.99996360706962</v>
+        <v>0</v>
       </c>
       <c r="N142" t="n">
-        <v>99.99996360706962</v>
+        <v>0</v>
       </c>
       <c r="O142" t="n">
-        <v>99.99996360706962</v>
+        <v>0</v>
       </c>
       <c r="P142" t="n">
         <v>7.848967307763466e-05</v>
       </c>
-      <c r="Q142" t="n">
-        <v>0.2919452869008161</v>
-      </c>
+      <c r="Q142" t="inlineStr"/>
       <c r="R142" t="n">
-        <v>0.005071203133966255</v>
+        <v>0.00392007475394973</v>
       </c>
       <c r="S142" t="n">
-        <v>0.00277129275109098</v>
+        <v>0.001990112621872396</v>
       </c>
       <c r="T142" t="n">
-        <v>0.0004973419972213941</v>
+        <v>9.486809831860035e-05</v>
       </c>
       <c r="U142" t="n">
-        <v>0.00436593221284905</v>
+        <v>0.003143283040122563</v>
       </c>
       <c r="V142" t="n">
         <v>34</v>
@@ -24977,38 +24931,36 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L143" t="n">
-        <v>78.68485143096366</v>
+        <v>99.99999442246379</v>
       </c>
       <c r="M143" t="n">
-        <v>78.68485143096366</v>
+        <v>0</v>
       </c>
       <c r="N143" t="n">
-        <v>78.68485143096366</v>
+        <v>0</v>
       </c>
       <c r="O143" t="n">
-        <v>78.68485143096366</v>
+        <v>0</v>
       </c>
       <c r="P143" t="n">
         <v>0.0001635415500933215</v>
       </c>
-      <c r="Q143" t="n">
-        <v>58043967.00968617</v>
-      </c>
+      <c r="Q143" t="inlineStr"/>
       <c r="R143" t="n">
-        <v>0.0103122108976768</v>
+        <v>0.007143808121774246</v>
       </c>
       <c r="S143" t="n">
-        <v>0.005442930061592062</v>
+        <v>0.003408817500397292</v>
       </c>
       <c r="T143" t="n">
-        <v>0.0008552971663018383</v>
+        <v>0.0005485123809050255</v>
       </c>
       <c r="U143" t="n">
-        <v>0.008585204343096483</v>
+        <v>0.005368819913262519</v>
       </c>
       <c r="V143" t="n">
         <v>34</v>
@@ -25059,38 +25011,36 @@
       </c>
       <c r="K144" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L144" t="n">
-        <v>38.52515852264099</v>
+        <v>0.006166637070935121</v>
       </c>
       <c r="M144" t="n">
-        <v>38.52515852264099</v>
+        <v>0</v>
       </c>
       <c r="N144" t="n">
-        <v>38.52515852264099</v>
+        <v>0</v>
       </c>
       <c r="O144" t="n">
-        <v>38.52515852264099</v>
+        <v>0</v>
       </c>
       <c r="P144" t="n">
         <v>3.753280708013851e-05</v>
       </c>
-      <c r="Q144" t="n">
-        <v>0.2432067289276859</v>
-      </c>
+      <c r="Q144" t="inlineStr"/>
       <c r="R144" t="n">
-        <v>0.002593839597142213</v>
+        <v>0.002442445064453101</v>
       </c>
       <c r="S144" t="n">
-        <v>0.001373217213489001</v>
+        <v>0.001270677376393683</v>
       </c>
       <c r="T144" t="n">
-        <v>0.0001008489705010066</v>
+        <v>2.562494254889063e-05</v>
       </c>
       <c r="U144" t="n">
-        <v>0.002168728924451103</v>
+        <v>0.002007540185029948</v>
       </c>
       <c r="V144" t="n">
         <v>34</v>
@@ -25223,38 +25173,36 @@
       </c>
       <c r="K146" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L146" t="n">
         <v>99.99982965062681</v>
       </c>
       <c r="M146" t="n">
-        <v>99.99982965062681</v>
+        <v>0</v>
       </c>
       <c r="N146" t="n">
-        <v>99.99982965062681</v>
+        <v>0</v>
       </c>
       <c r="O146" t="n">
-        <v>99.99982965062681</v>
+        <v>0</v>
       </c>
       <c r="P146" t="n">
         <v>2.921257405690759e-05</v>
       </c>
-      <c r="Q146" t="n">
-        <v>0.4838199195311653</v>
-      </c>
+      <c r="Q146" t="inlineStr"/>
       <c r="R146" t="n">
-        <v>0.001790366265953686</v>
+        <v>0.001614439763129629</v>
       </c>
       <c r="S146" t="n">
-        <v>0.0009460837864889542</v>
+        <v>0.0008273740537738369</v>
       </c>
       <c r="T146" t="n">
-        <v>9.260140100443397e-05</v>
+        <v>3.721015607047206e-05</v>
       </c>
       <c r="U146" t="n">
-        <v>0.001493613371025049</v>
+        <v>0.001307121018856324</v>
       </c>
       <c r="V146" t="n">
         <v>34</v>
@@ -25305,11 +25253,11 @@
       </c>
       <c r="K147" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L147" t="n">
-        <v>10.34958550447434</v>
+        <v>99.99999836563993</v>
       </c>
       <c r="M147" t="n">
         <v>0</v>
@@ -25323,9 +25271,7 @@
       <c r="P147" t="n">
         <v>3.938264210926682e-05</v>
       </c>
-      <c r="Q147" t="n">
-        <v>26269725.67056961</v>
-      </c>
+      <c r="Q147" t="inlineStr"/>
       <c r="R147" t="n">
         <v>0.002480124375580798</v>
       </c>
@@ -25551,38 +25497,36 @@
       </c>
       <c r="K150" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L150" t="n">
         <v>99.99801771045323</v>
       </c>
       <c r="M150" t="n">
-        <v>99.99801771045323</v>
+        <v>0</v>
       </c>
       <c r="N150" t="n">
-        <v>99.99801771045323</v>
+        <v>0</v>
       </c>
       <c r="O150" t="n">
-        <v>99.99801771045323</v>
+        <v>0</v>
       </c>
       <c r="P150" t="n">
         <v>1.420209271449045e-05</v>
       </c>
-      <c r="Q150" t="n">
-        <v>2469908.851115822</v>
-      </c>
+      <c r="Q150" t="inlineStr"/>
       <c r="R150" t="n">
-        <v>0.0008215888854591221</v>
+        <v>0.0007817314769607411</v>
       </c>
       <c r="S150" t="n">
-        <v>0.0004307418741004909</v>
+        <v>0.0004042827286834804</v>
       </c>
       <c r="T150" t="n">
-        <v>1.887292306433218e-05</v>
+        <v>1.887391897343444e-05</v>
       </c>
       <c r="U150" t="n">
-        <v>0.0006804619292039376</v>
+        <v>0.0006386167770636597</v>
       </c>
       <c r="V150" t="n">
         <v>34</v>
@@ -25791,38 +25735,36 @@
       </c>
       <c r="K153" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L153" t="n">
-        <v>99.99998493565828</v>
+        <v>0.0005116473984365655</v>
       </c>
       <c r="M153" t="n">
-        <v>99.99998493565828</v>
+        <v>0</v>
       </c>
       <c r="N153" t="n">
-        <v>99.99998493565828</v>
+        <v>0</v>
       </c>
       <c r="O153" t="n">
-        <v>99.99998493565828</v>
+        <v>0</v>
       </c>
       <c r="P153" t="n">
         <v>8.522180912716315e-06</v>
       </c>
-      <c r="Q153" t="n">
-        <v>4636390.631610394</v>
-      </c>
+      <c r="Q153" t="inlineStr"/>
       <c r="R153" t="n">
-        <v>0.0006500283924117827</v>
+        <v>0.0006246077017249942</v>
       </c>
       <c r="S153" t="n">
-        <v>0.0003443135722146441</v>
+        <v>0.000327816174634259</v>
       </c>
       <c r="T153" t="n">
-        <v>2.964000591648263e-05</v>
+        <v>3.783749483542175e-05</v>
       </c>
       <c r="U153" t="n">
-        <v>0.0005434317804474914</v>
+        <v>0.0005171450567757086</v>
       </c>
       <c r="V153" t="n">
         <v>34</v>
@@ -25873,38 +25815,36 @@
       </c>
       <c r="K154" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L154" t="n">
-        <v>99.99881055196656</v>
+        <v>99.23871421384499</v>
       </c>
       <c r="M154" t="n">
-        <v>99.99881055196656</v>
+        <v>0</v>
       </c>
       <c r="N154" t="n">
-        <v>99.99881055196656</v>
+        <v>0</v>
       </c>
       <c r="O154" t="n">
-        <v>99.99881055196656</v>
+        <v>0</v>
       </c>
       <c r="P154" t="n">
         <v>6.335042100090133e-06</v>
       </c>
-      <c r="Q154" t="n">
-        <v>3297662.181032485</v>
-      </c>
+      <c r="Q154" t="inlineStr"/>
       <c r="R154" t="n">
-        <v>0.0003846742011087939</v>
+        <v>0.0003757243948449169</v>
       </c>
       <c r="S154" t="n">
-        <v>0.0001953733419747284</v>
+        <v>0.0001896080617882982</v>
       </c>
       <c r="T154" t="n">
-        <v>1.244555220564182e-05</v>
+        <v>1.496445151053687e-05</v>
       </c>
       <c r="U154" t="n">
-        <v>0.0003085090956977543</v>
+        <v>0.0002993324262055668</v>
       </c>
       <c r="V154" t="n">
         <v>34</v>
@@ -25955,7 +25895,7 @@
       </c>
       <c r="K155" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L155" t="n">
@@ -25973,9 +25913,7 @@
       <c r="P155" t="n">
         <v>1.199127754394794e-05</v>
       </c>
-      <c r="Q155" t="n">
-        <v>11371255.20877764</v>
-      </c>
+      <c r="Q155" t="inlineStr"/>
       <c r="R155" t="n">
         <v>0.0003105253301246925</v>
       </c>
@@ -28497,38 +28435,36 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L186" t="n">
         <v>99.99999803708718</v>
       </c>
       <c r="M186" t="n">
-        <v>99.99999803708718</v>
+        <v>0</v>
       </c>
       <c r="N186" t="n">
-        <v>99.99999803708718</v>
+        <v>0</v>
       </c>
       <c r="O186" t="n">
-        <v>99.99999803708718</v>
+        <v>0</v>
       </c>
       <c r="P186" t="n">
         <v>2.938959455028546e-05</v>
       </c>
-      <c r="Q186" t="n">
-        <v>0.5091039728521236</v>
-      </c>
+      <c r="Q186" t="inlineStr"/>
       <c r="R186" t="n">
-        <v>0.001431397843017007</v>
+        <v>0.001320882144526264</v>
       </c>
       <c r="S186" t="n">
-        <v>0.0006671273655428144</v>
+        <v>0.0005956160331779327</v>
       </c>
       <c r="T186" t="n">
-        <v>6.558899011532143e-05</v>
+        <v>3.559526430164787e-05</v>
       </c>
       <c r="U186" t="n">
-        <v>0.001454792892308142</v>
+        <v>0.001299922129655748</v>
       </c>
       <c r="V186" t="n">
         <v>30</v>
@@ -28661,38 +28597,36 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L188" t="n">
-        <v>89.05825463352933</v>
+        <v>99.98618857108376</v>
       </c>
       <c r="M188" t="n">
-        <v>89.05825463352933</v>
+        <v>0</v>
       </c>
       <c r="N188" t="n">
-        <v>89.05825463352933</v>
+        <v>0</v>
       </c>
       <c r="O188" t="n">
-        <v>89.05825463352933</v>
+        <v>0</v>
       </c>
       <c r="P188" t="n">
         <v>1.580741089325414e-05</v>
       </c>
-      <c r="Q188" t="n">
-        <v>0.3590073916814031</v>
-      </c>
+      <c r="Q188" t="inlineStr"/>
       <c r="R188" t="n">
-        <v>0.0007914125089065911</v>
+        <v>0.0007593707413815071</v>
       </c>
       <c r="S188" t="n">
-        <v>0.0003769548897103433</v>
+        <v>0.0003551004861180686</v>
       </c>
       <c r="T188" t="n">
-        <v>4.648425192695484e-05</v>
+        <v>2.708959165528889e-05</v>
       </c>
       <c r="U188" t="n">
-        <v>0.0008211834407751577</v>
+        <v>0.0007744433956394527</v>
       </c>
       <c r="V188" t="n">
         <v>30</v>
@@ -28907,7 +28841,7 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L191" t="n">
@@ -28925,9 +28859,7 @@
       <c r="P191" t="n">
         <v>3.469442318178457e-05</v>
       </c>
-      <c r="Q191" t="n">
-        <v>29071139.37547025</v>
-      </c>
+      <c r="Q191" t="inlineStr"/>
       <c r="R191" t="n">
         <v>0.0007949568205817212</v>
       </c>
@@ -28989,38 +28921,36 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L192" t="n">
         <v>99.97344800904655</v>
       </c>
       <c r="M192" t="n">
-        <v>99.97344800904655</v>
+        <v>0</v>
       </c>
       <c r="N192" t="n">
-        <v>99.97344800904655</v>
+        <v>0</v>
       </c>
       <c r="O192" t="n">
-        <v>99.97344800904655</v>
+        <v>0</v>
       </c>
       <c r="P192" t="n">
         <v>8.817038345936803e-06</v>
       </c>
-      <c r="Q192" t="n">
-        <v>1.425028811651335</v>
-      </c>
+      <c r="Q192" t="inlineStr"/>
       <c r="R192" t="n">
-        <v>0.0004528462042830653</v>
+        <v>0.0004411151320676545</v>
       </c>
       <c r="S192" t="n">
-        <v>0.0001993373511043683</v>
+        <v>0.000192518908537091</v>
       </c>
       <c r="T192" t="n">
-        <v>2.468565308148623e-05</v>
+        <v>2.855324086729275e-05</v>
       </c>
       <c r="U192" t="n">
-        <v>0.0004343090977486118</v>
+        <v>0.0004191199943399665</v>
       </c>
       <c r="V192" t="n">
         <v>30</v>
@@ -29071,20 +29001,20 @@
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L193" t="n">
         <v>99.99503978336416</v>
       </c>
       <c r="M193" t="n">
-        <v>99.99503978336416</v>
+        <v>0</v>
       </c>
       <c r="N193" t="n">
-        <v>99.99503978336416</v>
+        <v>0</v>
       </c>
       <c r="O193" t="n">
-        <v>99.99503978336416</v>
+        <v>0</v>
       </c>
       <c r="P193" t="n">
         <v>6.633179880177407e-06</v>
@@ -29093,16 +29023,16 @@
         <v>2864696.635007625</v>
       </c>
       <c r="R193" t="n">
-        <v>0.0005132602183423087</v>
+        <v>0.0004981803842975393</v>
       </c>
       <c r="S193" t="n">
-        <v>0.0002297082577631935</v>
+        <v>0.0002210129608862976</v>
       </c>
       <c r="T193" t="n">
-        <v>3.233102494539539e-05</v>
+        <v>3.686210989349765e-05</v>
       </c>
       <c r="U193" t="n">
-        <v>0.0004999671133173038</v>
+        <v>0.0004805218915453714</v>
       </c>
       <c r="V193" t="n">
         <v>30</v>
@@ -29153,38 +29083,36 @@
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L194" t="n">
         <v>99.99372184353503</v>
       </c>
       <c r="M194" t="n">
-        <v>99.99372184353503</v>
+        <v>0</v>
       </c>
       <c r="N194" t="n">
-        <v>99.99372184353503</v>
+        <v>0</v>
       </c>
       <c r="O194" t="n">
-        <v>99.99372184353503</v>
+        <v>0</v>
       </c>
       <c r="P194" t="n">
         <v>6.999245188682134e-06</v>
       </c>
-      <c r="Q194" t="n">
-        <v>3570851.499325457</v>
-      </c>
+      <c r="Q194" t="inlineStr"/>
       <c r="R194" t="n">
-        <v>0.0003060142813247015</v>
+        <v>0.0003005821327928658</v>
       </c>
       <c r="S194" t="n">
-        <v>0.0001356547567954825</v>
+        <v>0.0001323624927501625</v>
       </c>
       <c r="T194" t="n">
-        <v>1.122076225070992e-05</v>
+        <v>1.17334467738004e-05</v>
       </c>
       <c r="U194" t="n">
-        <v>0.0002958636339762149</v>
+        <v>0.0002886097740778493</v>
       </c>
       <c r="V194" t="n">
         <v>30</v>
@@ -29311,20 +29239,20 @@
       </c>
       <c r="K196" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L196" t="n">
         <v>99.96015548986463</v>
       </c>
       <c r="M196" t="n">
-        <v>99.96015548986463</v>
+        <v>0</v>
       </c>
       <c r="N196" t="n">
-        <v>99.96015548986463</v>
+        <v>0</v>
       </c>
       <c r="O196" t="n">
-        <v>99.96015548986463</v>
+        <v>0</v>
       </c>
       <c r="P196" t="n">
         <v>4.079953198282405e-06</v>
@@ -29333,16 +29261,16 @@
         <v>2114622.310700125</v>
       </c>
       <c r="R196" t="n">
-        <v>0.0002264759587083437</v>
+        <v>0.0002234323104801488</v>
       </c>
       <c r="S196" t="n">
-        <v>0.0001056422134585498</v>
+        <v>0.0001036889507377813</v>
       </c>
       <c r="T196" t="n">
-        <v>7.284155627157517e-06</v>
+        <v>7.601530683317884e-06</v>
       </c>
       <c r="U196" t="n">
-        <v>0.0002304746802467088</v>
+        <v>0.0002262147439890981</v>
       </c>
       <c r="V196" t="n">
         <v>30</v>
@@ -31853,20 +31781,20 @@
       </c>
       <c r="K227" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L227" t="n">
         <v>99.99999971390291</v>
       </c>
       <c r="M227" t="n">
-        <v>99.99999971390291</v>
+        <v>0</v>
       </c>
       <c r="N227" t="n">
-        <v>99.99999971390291</v>
+        <v>0</v>
       </c>
       <c r="O227" t="n">
-        <v>99.99999971390291</v>
+        <v>0</v>
       </c>
       <c r="P227" t="n">
         <v>6.772917316486888e-05</v>
@@ -31875,16 +31803,16 @@
         <v>0.2206651855977209</v>
       </c>
       <c r="R227" t="n">
-        <v>0.002327046401312462</v>
+        <v>0.002037488448961765</v>
       </c>
       <c r="S227" t="n">
-        <v>0.001320674793648838</v>
+        <v>0.001060488932150703</v>
       </c>
       <c r="T227" t="n">
-        <v>0.0001472408954395488</v>
+        <v>7.487557460020175e-05</v>
       </c>
       <c r="U227" t="n">
-        <v>0.003760740443133564</v>
+        <v>0.003024498178451425</v>
       </c>
       <c r="V227" t="n">
         <v>30</v>
@@ -31935,38 +31863,36 @@
       </c>
       <c r="K228" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L228" t="n">
-        <v>99.99999999000001</v>
+        <v>99.99999999992984</v>
       </c>
       <c r="M228" t="n">
-        <v>99.99999999000001</v>
+        <v>0</v>
       </c>
       <c r="N228" t="n">
-        <v>99.99999999000001</v>
+        <v>0</v>
       </c>
       <c r="O228" t="n">
-        <v>99.99999999000001</v>
+        <v>0</v>
       </c>
       <c r="P228" t="n">
         <v>0.000170992578460419</v>
       </c>
-      <c r="Q228" t="n">
-        <v>70390850.09955239</v>
-      </c>
+      <c r="Q228" t="inlineStr"/>
       <c r="R228" t="n">
-        <v>0.004997297509286166</v>
+        <v>0.003908974465295457</v>
       </c>
       <c r="S228" t="n">
-        <v>0.002548711816751884</v>
+        <v>0.001746186479157552</v>
       </c>
       <c r="T228" t="n">
-        <v>0.0005411242033192985</v>
+        <v>0.0006925524551776896</v>
       </c>
       <c r="U228" t="n">
-        <v>0.007240936048058419</v>
+        <v>0.00490906086153269</v>
       </c>
       <c r="V228" t="n">
         <v>30</v>
@@ -32017,38 +31943,36 @@
       </c>
       <c r="K229" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L229" t="n">
         <v>99.99999341688996</v>
       </c>
       <c r="M229" t="n">
-        <v>99.99999341688996</v>
+        <v>0</v>
       </c>
       <c r="N229" t="n">
-        <v>99.99999341688996</v>
+        <v>0</v>
       </c>
       <c r="O229" t="n">
-        <v>99.99999341688996</v>
+        <v>0</v>
       </c>
       <c r="P229" t="n">
         <v>4.783315080175279e-05</v>
       </c>
-      <c r="Q229" t="n">
-        <v>0.3504693534553042</v>
-      </c>
+      <c r="Q229" t="inlineStr"/>
       <c r="R229" t="n">
-        <v>0.001519522650235268</v>
+        <v>0.00138819057162991</v>
       </c>
       <c r="S229" t="n">
-        <v>0.000857356434479111</v>
+        <v>0.0007367977815809061</v>
       </c>
       <c r="T229" t="n">
-        <v>9.982308602006669e-05</v>
+        <v>3.213355731554804e-05</v>
       </c>
       <c r="U229" t="n">
-        <v>0.002441836229918237</v>
+        <v>0.002101987964528366</v>
       </c>
       <c r="V229" t="n">
         <v>30</v>
@@ -32099,38 +32023,36 @@
       </c>
       <c r="K230" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L230" t="n">
-        <v>19.81185314384397</v>
+        <v>25.38225861862774</v>
       </c>
       <c r="M230" t="n">
-        <v>19.81185314384397</v>
+        <v>0</v>
       </c>
       <c r="N230" t="n">
-        <v>19.81185314384397</v>
+        <v>0</v>
       </c>
       <c r="O230" t="n">
-        <v>19.81185314384397</v>
+        <v>0</v>
       </c>
       <c r="P230" t="n">
         <v>3.406160417725151e-05</v>
       </c>
-      <c r="Q230" t="n">
-        <v>0.2340683620106587</v>
-      </c>
+      <c r="Q230" t="inlineStr"/>
       <c r="R230" t="n">
-        <v>0.00111307356336778</v>
+        <v>0.001097408926170615</v>
       </c>
       <c r="S230" t="n">
-        <v>0.0006248951510910768</v>
+        <v>0.0006101041734515625</v>
       </c>
       <c r="T230" t="n">
-        <v>5.324924377530638e-05</v>
+        <v>4.396469172088592e-05</v>
       </c>
       <c r="U230" t="n">
-        <v>0.001781255979998825</v>
+        <v>0.001739627484950403</v>
       </c>
       <c r="V230" t="n">
         <v>30</v>
@@ -32263,38 +32185,36 @@
       </c>
       <c r="K232" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L232" t="n">
         <v>99.99994153729666</v>
       </c>
       <c r="M232" t="n">
-        <v>99.99994153729666</v>
+        <v>0</v>
       </c>
       <c r="N232" t="n">
-        <v>99.99994153729666</v>
+        <v>0</v>
       </c>
       <c r="O232" t="n">
-        <v>99.99994153729666</v>
+        <v>0</v>
       </c>
       <c r="P232" t="n">
         <v>3.602800973964414e-05</v>
       </c>
-      <c r="Q232" t="n">
-        <v>0.7614451852772578</v>
-      </c>
+      <c r="Q232" t="inlineStr"/>
       <c r="R232" t="n">
-        <v>0.0008932060210565528</v>
+        <v>0.0008457799193493762</v>
       </c>
       <c r="S232" t="n">
-        <v>0.0004917530180698051</v>
+        <v>0.0004485286151283934</v>
       </c>
       <c r="T232" t="n">
-        <v>6.174881707856969e-05</v>
+        <v>3.76430938859606e-05</v>
       </c>
       <c r="U232" t="n">
-        <v>0.001401328722750151</v>
+        <v>0.001279295396406319</v>
       </c>
       <c r="V232" t="n">
         <v>30</v>
@@ -32345,11 +32265,11 @@
       </c>
       <c r="K233" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L233" t="n">
-        <v>52.07399938339263</v>
+        <v>73.26228302528797</v>
       </c>
       <c r="M233" t="n">
         <v>0</v>
@@ -32363,9 +32283,7 @@
       <c r="P233" t="n">
         <v>5.345341205086612e-05</v>
       </c>
-      <c r="Q233" t="n">
-        <v>32735972.06057775</v>
-      </c>
+      <c r="Q233" t="inlineStr"/>
       <c r="R233" t="n">
         <v>0.001833380486925216</v>
       </c>
@@ -32427,38 +32345,36 @@
       </c>
       <c r="K234" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L234" t="n">
         <v>99.996277246481</v>
       </c>
       <c r="M234" t="n">
-        <v>99.996277246481</v>
+        <v>0</v>
       </c>
       <c r="N234" t="n">
-        <v>99.996277246481</v>
+        <v>0</v>
       </c>
       <c r="O234" t="n">
-        <v>99.996277246481</v>
+        <v>0</v>
       </c>
       <c r="P234" t="n">
         <v>1.704503059737354e-05</v>
       </c>
-      <c r="Q234" t="n">
-        <v>0.4759636511517844</v>
-      </c>
+      <c r="Q234" t="inlineStr"/>
       <c r="R234" t="n">
-        <v>0.0005294230423122233</v>
+        <v>0.0005120772961609127</v>
       </c>
       <c r="S234" t="n">
-        <v>0.0002965110092956001</v>
+        <v>0.0002802444165488555</v>
       </c>
       <c r="T234" t="n">
-        <v>3.145345981249859e-05</v>
+        <v>2.132992279347656e-05</v>
       </c>
       <c r="U234" t="n">
-        <v>0.0008447921562627742</v>
+        <v>0.0007990325478955438</v>
       </c>
       <c r="V234" t="n">
         <v>30</v>
@@ -32509,38 +32425,36 @@
       </c>
       <c r="K235" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L235" t="n">
         <v>99.98669975490962</v>
       </c>
       <c r="M235" t="n">
-        <v>99.98669975490962</v>
+        <v>0</v>
       </c>
       <c r="N235" t="n">
-        <v>99.98669975490962</v>
+        <v>0</v>
       </c>
       <c r="O235" t="n">
-        <v>99.98669975490962</v>
+        <v>0</v>
       </c>
       <c r="P235" t="n">
         <v>1.431342172750345e-05</v>
       </c>
-      <c r="Q235" t="n">
-        <v>2626426.816829497</v>
-      </c>
+      <c r="Q235" t="inlineStr"/>
       <c r="R235" t="n">
-        <v>0.000469977757212239</v>
+        <v>0.0004562358103491702</v>
       </c>
       <c r="S235" t="n">
-        <v>0.0002632117076737572</v>
+        <v>0.0002501407978425201</v>
       </c>
       <c r="T235" t="n">
-        <v>2.762447331015348e-05</v>
+        <v>1.973946493678862e-05</v>
       </c>
       <c r="U235" t="n">
-        <v>0.0007494113835341903</v>
+        <v>0.0007128262705269853</v>
       </c>
       <c r="V235" t="n">
         <v>30</v>
@@ -32591,38 +32505,36 @@
       </c>
       <c r="K236" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L236" t="n">
-        <v>99.99999999000001</v>
+        <v>99.99999999483958</v>
       </c>
       <c r="M236" t="n">
-        <v>99.99999999000001</v>
+        <v>0</v>
       </c>
       <c r="N236" t="n">
-        <v>99.99999999000001</v>
+        <v>0</v>
       </c>
       <c r="O236" t="n">
-        <v>99.99999999000001</v>
+        <v>0</v>
       </c>
       <c r="P236" t="n">
         <v>7.414931569872714e-05</v>
       </c>
-      <c r="Q236" t="n">
-        <v>38198811.96757618</v>
-      </c>
+      <c r="Q236" t="inlineStr"/>
       <c r="R236" t="n">
-        <v>0.00155645156276854</v>
+        <v>0.001424851037876168</v>
       </c>
       <c r="S236" t="n">
-        <v>0.000772656986167189</v>
+        <v>0.0006719607183687834</v>
       </c>
       <c r="T236" t="n">
-        <v>0.0002008288639484539</v>
+        <v>0.0001759775948256653</v>
       </c>
       <c r="U236" t="n">
-        <v>0.002190780829347365</v>
+        <v>0.001899105134438318</v>
       </c>
       <c r="V236" t="n">
         <v>30</v>
@@ -32673,38 +32585,36 @@
       </c>
       <c r="K237" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L237" t="n">
         <v>99.99999916573678</v>
       </c>
       <c r="M237" t="n">
-        <v>99.99999916573678</v>
+        <v>0</v>
       </c>
       <c r="N237" t="n">
-        <v>99.99999916573678</v>
+        <v>0</v>
       </c>
       <c r="O237" t="n">
-        <v>99.99999916573678</v>
+        <v>0</v>
       </c>
       <c r="P237" t="n">
         <v>1.687295514046056e-05</v>
       </c>
-      <c r="Q237" t="n">
-        <v>3076397.474506717</v>
-      </c>
+      <c r="Q237" t="inlineStr"/>
       <c r="R237" t="n">
-        <v>0.0004454153653581254</v>
+        <v>0.000433364620988219</v>
       </c>
       <c r="S237" t="n">
-        <v>0.0002337445164542082</v>
+        <v>0.0002234939958973909</v>
       </c>
       <c r="T237" t="n">
-        <v>1.66644782261631e-05</v>
+        <v>1.835722626385421e-05</v>
       </c>
       <c r="U237" t="n">
-        <v>0.000666705311783686</v>
+        <v>0.0006372878074706399</v>
       </c>
       <c r="V237" t="n">
         <v>30</v>
@@ -32831,38 +32741,36 @@
       </c>
       <c r="K239" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L239" t="n">
         <v>99.99525725585139</v>
       </c>
       <c r="M239" t="n">
-        <v>99.99525725585139</v>
+        <v>0</v>
       </c>
       <c r="N239" t="n">
-        <v>99.99525725585139</v>
+        <v>0</v>
       </c>
       <c r="O239" t="n">
-        <v>99.99525725585139</v>
+        <v>0</v>
       </c>
       <c r="P239" t="n">
         <v>9.229630940260271e-06</v>
       </c>
-      <c r="Q239" t="n">
-        <v>1688692.847637749</v>
-      </c>
+      <c r="Q239" t="inlineStr"/>
       <c r="R239" t="n">
-        <v>0.0002753673085496699</v>
+        <v>0.0002707718845250956</v>
       </c>
       <c r="S239" t="n">
-        <v>0.0001380828465564839</v>
+        <v>0.0001343441064065541</v>
       </c>
       <c r="T239" t="n">
-        <v>1.537318350576018e-05</v>
+        <v>1.57995486963074e-05</v>
       </c>
       <c r="U239" t="n">
-        <v>0.0003935623537089095</v>
+        <v>0.0003827735474522296</v>
       </c>
       <c r="V239" t="n">
         <v>30</v>
@@ -32913,20 +32821,20 @@
       </c>
       <c r="K240" t="inlineStr">
         <is>
-          <t>ok</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L240" t="n">
         <v>99.99979978102513</v>
       </c>
       <c r="M240" t="n">
-        <v>99.99979978102513</v>
+        <v>0</v>
       </c>
       <c r="N240" t="n">
-        <v>99.99979978102513</v>
+        <v>0</v>
       </c>
       <c r="O240" t="n">
-        <v>99.99979978102513</v>
+        <v>0</v>
       </c>
       <c r="P240" t="n">
         <v>7.360196266000505e-06</v>
@@ -32935,16 +32843,16 @@
         <v>2770403.084891323</v>
       </c>
       <c r="R240" t="n">
-        <v>0.000318983591557863</v>
+        <v>0.0003128303553876498</v>
       </c>
       <c r="S240" t="n">
-        <v>0.000160514255764453</v>
+        <v>0.0001557457448983109</v>
       </c>
       <c r="T240" t="n">
-        <v>2.913910356226763e-05</v>
+        <v>3.185940818841628e-05</v>
       </c>
       <c r="U240" t="n">
-        <v>0.0004562637752503819</v>
+        <v>0.0004422953356516692</v>
       </c>
       <c r="V240" t="n">
         <v>30</v>
@@ -32995,7 +32903,7 @@
       </c>
       <c r="K241" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L241" t="n">
@@ -33013,9 +32921,7 @@
       <c r="P241" t="n">
         <v>2.395439085816805e-05</v>
       </c>
-      <c r="Q241" t="n">
-        <v>21751739.7452101</v>
-      </c>
+      <c r="Q241" t="inlineStr"/>
       <c r="R241" t="n">
         <v>0.0006869516033407636</v>
       </c>
@@ -33235,38 +33141,36 @@
       </c>
       <c r="K244" t="inlineStr">
         <is>
-          <t>delta_inapplicable</t>
+          <t>insufficient_signal</t>
         </is>
       </c>
       <c r="L244" t="n">
         <v>99.99923978474666</v>
       </c>
       <c r="M244" t="n">
-        <v>99.99923978474666</v>
+        <v>0</v>
       </c>
       <c r="N244" t="n">
-        <v>99.99923978474666</v>
+        <v>0</v>
       </c>
       <c r="O244" t="n">
-        <v>99.99923978474666</v>
+        <v>0</v>
       </c>
       <c r="P244" t="n">
         <v>6.036354065552406e-06</v>
       </c>
-      <c r="Q244" t="n">
-        <v>3431271.645127978</v>
-      </c>
+      <c r="Q244" t="inlineStr"/>
       <c r="R244" t="n">
-        <v>0.0001415070945738624</v>
+        <v>0.0001402356264045068</v>
       </c>
       <c r="S244" t="n">
-        <v>7.718264970584943e-05</v>
+        <v>7.603702586640407e-05</v>
       </c>
       <c r="T244" t="n">
-        <v>9.776568936260753e-06</v>
+        <v>9.137998758798719e-06</v>
       </c>
       <c r="U244" t="n">
-        <v>0.0002199269314165493</v>
+        <v>0.0002166707483838106</v>
       </c>
       <c r="V244" t="n">
         <v>30</v>

</xml_diff>

<commit_message>
version 7.6 with PROPER NPH correction based on alpha from config file. Ready to run!
</commit_message>
<xml_diff>
--- a/data/Czech/KCOR_summary.xlsx
+++ b/data/Czech/KCOR_summary.xlsx
@@ -540,17 +540,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1.2066</t>
+          <t>1.1567</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.181</t>
+          <t>1.132</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.233</t>
+          <t>1.182</t>
         </is>
       </c>
       <c r="F4" t="b">
@@ -581,17 +581,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1.0161</t>
+          <t>0.9509</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.934</t>
+          <t>0.875</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.105</t>
+          <t>1.034</t>
         </is>
       </c>
       <c r="F5" t="b">
@@ -622,17 +622,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1.0134</t>
+          <t>0.9581</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.973</t>
+          <t>0.920</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.056</t>
+          <t>0.998</t>
         </is>
       </c>
       <c r="F6" t="b">
@@ -663,17 +663,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1.4317</t>
+          <t>1.3659</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.388</t>
+          <t>1.325</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.477</t>
+          <t>1.408</t>
         </is>
       </c>
       <c r="F7" t="b">
@@ -704,17 +704,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1.4896</t>
+          <t>1.4484</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.377</t>
+          <t>1.339</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.612</t>
+          <t>1.567</t>
         </is>
       </c>
       <c r="F8" t="b">
@@ -745,17 +745,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.3231</t>
+          <t>1.2750</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.142</t>
+          <t>1.101</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.532</t>
+          <t>1.476</t>
         </is>
       </c>
       <c r="F9" t="b">
@@ -786,17 +786,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2.9678</t>
+          <t>2.8393</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.330</t>
+          <t>2.230</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.780</t>
+          <t>3.616</t>
         </is>
       </c>
       <c r="F10" t="b">
@@ -827,17 +827,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.0879</t>
+          <t>1.0317</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.713</t>
+          <t>0.676</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.660</t>
+          <t>1.574</t>
         </is>
       </c>
       <c r="F11" t="b">
@@ -868,17 +868,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.3549</t>
+          <t>2.2365</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.402</t>
+          <t>1.334</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>3.954</t>
+          <t>3.751</t>
         </is>
       </c>
       <c r="F12" t="b">
@@ -909,17 +909,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12.6752</t>
+          <t>12.4845</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>5.962</t>
+          <t>5.875</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>26.946</t>
+          <t>26.530</t>
         </is>
       </c>
       <c r="F13" t="b">
@@ -984,17 +984,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1.4421</t>
+          <t>1.3824</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.419</t>
+          <t>1.360</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.466</t>
+          <t>1.405</t>
         </is>
       </c>
       <c r="F16" t="b">
@@ -1025,17 +1025,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1.3571</t>
+          <t>1.2700</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.297</t>
+          <t>1.216</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.420</t>
+          <t>1.327</t>
         </is>
       </c>
       <c r="F17" t="b">
@@ -1066,17 +1066,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.4686</t>
+          <t>1.3886</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.432</t>
+          <t>1.355</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.506</t>
+          <t>1.423</t>
         </is>
       </c>
       <c r="F18" t="b">
@@ -1107,17 +1107,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1.4929</t>
+          <t>1.4243</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.437</t>
+          <t>1.371</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.551</t>
+          <t>1.480</t>
         </is>
       </c>
       <c r="F19" t="b">
@@ -1148,17 +1148,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1.2339</t>
+          <t>1.1997</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.151</t>
+          <t>1.119</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.323</t>
+          <t>1.286</t>
         </is>
       </c>
       <c r="F20" t="b">
@@ -1189,17 +1189,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.2004</t>
+          <t>1.1567</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.038</t>
+          <t>1.001</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.388</t>
+          <t>1.337</t>
         </is>
       </c>
       <c r="F21" t="b">
@@ -1230,17 +1230,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.0975</t>
+          <t>1.0500</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.864</t>
+          <t>0.827</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.395</t>
+          <t>1.334</t>
         </is>
       </c>
       <c r="F22" t="b">
@@ -1271,17 +1271,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.6309</t>
+          <t>0.5983</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.409</t>
+          <t>0.388</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0.974</t>
+          <t>0.924</t>
         </is>
       </c>
       <c r="F23" t="b">
@@ -1312,17 +1312,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1.2510</t>
+          <t>1.1881</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.746</t>
+          <t>0.709</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2.099</t>
+          <t>1.991</t>
         </is>
       </c>
       <c r="F24" t="b">
@@ -1353,17 +1353,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2.2822</t>
+          <t>2.2478</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.320</t>
+          <t>0.315</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>16.279</t>
+          <t>16.031</t>
         </is>
       </c>
       <c r="F25" t="b">
@@ -1962,17 +1962,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1.1850</t>
+          <t>1.1305</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1.162</t>
+          <t>1.109</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.208</t>
+          <t>1.152</t>
         </is>
       </c>
       <c r="F4" t="b">
@@ -2003,17 +2003,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.7970</t>
+          <t>0.7497</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.725</t>
+          <t>0.682</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.876</t>
+          <t>0.824</t>
         </is>
       </c>
       <c r="F5" t="b">
@@ -2044,17 +2044,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>1.0364</t>
+          <t>0.9737</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.985</t>
+          <t>0.926</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.090</t>
+          <t>1.024</t>
         </is>
       </c>
       <c r="F6" t="b">
@@ -2085,17 +2085,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1.0937</t>
+          <t>1.0447</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.057</t>
+          <t>1.010</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.131</t>
+          <t>1.080</t>
         </is>
       </c>
       <c r="F7" t="b">
@@ -2126,17 +2126,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1.4863</t>
+          <t>1.4261</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.437</t>
+          <t>1.379</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.538</t>
+          <t>1.475</t>
         </is>
       </c>
       <c r="F8" t="b">
@@ -2167,17 +2167,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.4266</t>
+          <t>1.3663</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.342</t>
+          <t>1.286</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.516</t>
+          <t>1.451</t>
         </is>
       </c>
       <c r="F9" t="b">
@@ -2208,17 +2208,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1.2429</t>
+          <t>1.1983</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.105</t>
+          <t>1.066</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.398</t>
+          <t>1.347</t>
         </is>
       </c>
       <c r="F10" t="b">
@@ -2249,17 +2249,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.2066</t>
+          <t>1.1406</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.948</t>
+          <t>0.897</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.536</t>
+          <t>1.451</t>
         </is>
       </c>
       <c r="F11" t="b">
@@ -2290,17 +2290,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.0902</t>
+          <t>1.0243</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.660</t>
+          <t>0.621</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.801</t>
+          <t>1.689</t>
         </is>
       </c>
       <c r="F12" t="b">
@@ -2331,17 +2331,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>7.3475</t>
+          <t>7.2631</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>4.013</t>
+          <t>3.968</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>13.454</t>
+          <t>13.294</t>
         </is>
       </c>
       <c r="F13" t="b">
@@ -2406,17 +2406,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1.1262</t>
+          <t>1.0744</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.110</t>
+          <t>1.060</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.142</t>
+          <t>1.090</t>
         </is>
       </c>
       <c r="F16" t="b">
@@ -2447,17 +2447,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1.0236</t>
+          <t>0.9628</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.979</t>
+          <t>0.922</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.070</t>
+          <t>1.005</t>
         </is>
       </c>
       <c r="F17" t="b">
@@ -2488,17 +2488,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.0691</t>
+          <t>1.0045</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.042</t>
+          <t>0.980</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.097</t>
+          <t>1.029</t>
         </is>
       </c>
       <c r="F18" t="b">
@@ -2529,17 +2529,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1.2794</t>
+          <t>1.2221</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.247</t>
+          <t>1.192</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.313</t>
+          <t>1.253</t>
         </is>
       </c>
       <c r="F19" t="b">
@@ -2570,17 +2570,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1.0898</t>
+          <t>1.0457</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.038</t>
+          <t>0.996</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.144</t>
+          <t>1.098</t>
         </is>
       </c>
       <c r="F20" t="b">
@@ -2611,17 +2611,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.2368</t>
+          <t>1.1845</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.125</t>
+          <t>1.078</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.359</t>
+          <t>1.301</t>
         </is>
       </c>
       <c r="F21" t="b">
@@ -2652,17 +2652,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.0287</t>
+          <t>0.9918</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.884</t>
+          <t>0.853</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.197</t>
+          <t>1.154</t>
         </is>
       </c>
       <c r="F22" t="b">
@@ -2693,17 +2693,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2.7903</t>
+          <t>2.6376</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.181</t>
+          <t>2.064</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3.570</t>
+          <t>3.371</t>
         </is>
       </c>
       <c r="F23" t="b">
@@ -2734,17 +2734,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.9048</t>
+          <t>0.8501</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.641</t>
+          <t>0.603</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.278</t>
+          <t>1.198</t>
         </is>
       </c>
       <c r="F24" t="b">
@@ -2775,17 +2775,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>6.8041</t>
+          <t>6.7260</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>3.490</t>
+          <t>3.451</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>13.267</t>
+          <t>13.110</t>
         </is>
       </c>
       <c r="F25" t="b">
@@ -3384,17 +3384,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.9902</t>
+          <t>0.9411</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.968</t>
+          <t>0.921</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>1.012</t>
+          <t>0.962</t>
         </is>
       </c>
       <c r="F4" t="b">
@@ -3425,17 +3425,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.7803</t>
+          <t>0.7375</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.692</t>
+          <t>0.655</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.880</t>
+          <t>0.831</t>
         </is>
       </c>
       <c r="F5" t="b">
@@ -3466,17 +3466,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.9529</t>
+          <t>0.8905</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.901</t>
+          <t>0.843</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.007</t>
+          <t>0.941</t>
         </is>
       </c>
       <c r="F6" t="b">
@@ -3507,17 +3507,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.9148</t>
+          <t>0.8708</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.876</t>
+          <t>0.834</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.956</t>
+          <t>0.909</t>
         </is>
       </c>
       <c r="F7" t="b">
@@ -3548,17 +3548,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1.1362</t>
+          <t>1.0864</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.091</t>
+          <t>1.043</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.184</t>
+          <t>1.131</t>
         </is>
       </c>
       <c r="F8" t="b">
@@ -3589,17 +3589,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.1384</t>
+          <t>1.0885</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.073</t>
+          <t>1.027</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.208</t>
+          <t>1.154</t>
         </is>
       </c>
       <c r="F9" t="b">
@@ -3630,17 +3630,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1.2451</t>
+          <t>1.1995</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.139</t>
+          <t>1.098</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.361</t>
+          <t>1.310</t>
         </is>
       </c>
       <c r="F10" t="b">
@@ -3671,17 +3671,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.0103</t>
+          <t>0.9668</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.847</t>
+          <t>0.812</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.205</t>
+          <t>1.151</t>
         </is>
       </c>
       <c r="F11" t="b">
@@ -3712,17 +3712,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3.4186</t>
+          <t>3.1828</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2.435</t>
+          <t>2.274</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>4.800</t>
+          <t>4.455</t>
         </is>
       </c>
       <c r="F12" t="b">
@@ -3753,17 +3753,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>0.5954</t>
+          <t>0.5841</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.306</t>
+          <t>0.300</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.158</t>
+          <t>1.135</t>
         </is>
       </c>
       <c r="F13" t="b">
@@ -3828,17 +3828,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1.0807</t>
+          <t>1.0271</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.066</t>
+          <t>1.014</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>1.095</t>
+          <t>1.041</t>
         </is>
       </c>
       <c r="F16" t="b">
@@ -3869,17 +3869,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1.0309</t>
+          <t>0.9744</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.983</t>
+          <t>0.931</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.081</t>
+          <t>1.020</t>
         </is>
       </c>
       <c r="F17" t="b">
@@ -3910,17 +3910,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.0212</t>
+          <t>0.9543</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.995</t>
+          <t>0.931</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.048</t>
+          <t>0.978</t>
         </is>
       </c>
       <c r="F18" t="b">
@@ -3951,17 +3951,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1.1195</t>
+          <t>1.0657</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
+          <t>1.040</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
           <t>1.092</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>1.147</t>
         </is>
       </c>
       <c r="F19" t="b">
@@ -3992,17 +3992,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1.3467</t>
+          <t>1.2876</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.301</t>
+          <t>1.245</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.394</t>
+          <t>1.332</t>
         </is>
       </c>
       <c r="F20" t="b">
@@ -4033,17 +4033,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.0854</t>
+          <t>1.0379</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.013</t>
+          <t>0.969</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.163</t>
+          <t>1.112</t>
         </is>
       </c>
       <c r="F21" t="b">
@@ -4074,17 +4074,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.1198</t>
+          <t>1.0787</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1.000</t>
+          <t>0.964</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.253</t>
+          <t>1.207</t>
         </is>
       </c>
       <c r="F22" t="b">
@@ -4115,17 +4115,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.3660</t>
+          <t>1.3071</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.115</t>
+          <t>1.068</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>1.674</t>
+          <t>1.600</t>
         </is>
       </c>
       <c r="F23" t="b">
@@ -4156,17 +4156,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>2.1371</t>
+          <t>1.9897</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1.556</t>
+          <t>1.453</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>2.936</t>
+          <t>2.724</t>
         </is>
       </c>
       <c r="F24" t="b">
@@ -4197,17 +4197,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.9749</t>
+          <t>0.9564</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.586</t>
+          <t>0.575</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>1.622</t>
+          <t>1.590</t>
         </is>
       </c>
       <c r="F25" t="b">
@@ -4806,17 +4806,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.7436</t>
+          <t>0.7046</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0.719</t>
+          <t>0.681</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.769</t>
+          <t>0.729</t>
         </is>
       </c>
       <c r="F4" t="b">
@@ -4847,17 +4847,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.5278</t>
+          <t>0.4983</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.438</t>
+          <t>0.413</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.637</t>
+          <t>0.601</t>
         </is>
       </c>
       <c r="F5" t="b">
@@ -4888,17 +4888,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.7267</t>
+          <t>0.6796</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.673</t>
+          <t>0.630</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.785</t>
+          <t>0.733</t>
         </is>
       </c>
       <c r="F6" t="b">
@@ -4929,17 +4929,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.6172</t>
+          <t>0.5852</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.573</t>
+          <t>0.544</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.665</t>
+          <t>0.630</t>
         </is>
       </c>
       <c r="F7" t="b">
@@ -4970,17 +4970,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.6433</t>
+          <t>0.6148</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.595</t>
+          <t>0.569</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.695</t>
+          <t>0.665</t>
         </is>
       </c>
       <c r="F8" t="b">
@@ -5011,17 +5011,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.9728</t>
+          <t>0.9279</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.871</t>
+          <t>0.831</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.086</t>
+          <t>1.036</t>
         </is>
       </c>
       <c r="F9" t="b">
@@ -5052,17 +5052,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1.0787</t>
+          <t>1.0309</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.931</t>
+          <t>0.891</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.250</t>
+          <t>1.193</t>
         </is>
       </c>
       <c r="F10" t="b">
@@ -5093,17 +5093,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.2307</t>
+          <t>1.1718</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.999</t>
+          <t>0.952</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.516</t>
+          <t>1.442</t>
         </is>
       </c>
       <c r="F11" t="b">
@@ -5134,17 +5134,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.0784</t>
+          <t>1.0149</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>0.786</t>
+          <t>0.742</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.480</t>
+          <t>1.388</t>
         </is>
       </c>
       <c r="F12" t="b">
@@ -5175,17 +5175,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1.2371</t>
+          <t>1.1818</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>0.839</t>
+          <t>0.803</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.825</t>
+          <t>1.738</t>
         </is>
       </c>
       <c r="F13" t="b">
@@ -5250,17 +5250,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.9653</t>
+          <t>0.9146</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>0.953</t>
+          <t>0.903</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>0.978</t>
+          <t>0.926</t>
         </is>
       </c>
       <c r="F16" t="b">
@@ -5291,17 +5291,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.9364</t>
+          <t>0.8840</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.893</t>
+          <t>0.844</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>0.982</t>
+          <t>0.926</t>
         </is>
       </c>
       <c r="F17" t="b">
@@ -5332,17 +5332,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.9062</t>
+          <t>0.8475</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.883</t>
+          <t>0.826</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0.930</t>
+          <t>0.869</t>
         </is>
       </c>
       <c r="F18" t="b">
@@ -5373,17 +5373,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.9785</t>
+          <t>0.9278</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.955</t>
+          <t>0.906</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.003</t>
+          <t>0.950</t>
         </is>
       </c>
       <c r="F19" t="b">
@@ -5414,17 +5414,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.9889</t>
+          <t>0.9452</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.959</t>
+          <t>0.917</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.020</t>
+          <t>0.974</t>
         </is>
       </c>
       <c r="F20" t="b">
@@ -5455,17 +5455,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.2945</t>
+          <t>1.2347</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.232</t>
+          <t>1.176</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.360</t>
+          <t>1.296</t>
         </is>
       </c>
       <c r="F21" t="b">
@@ -5496,17 +5496,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.1196</t>
+          <t>1.0700</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>1.037</t>
+          <t>0.992</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.209</t>
+          <t>1.154</t>
         </is>
       </c>
       <c r="F22" t="b">
@@ -5537,17 +5537,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1.7405</t>
+          <t>1.6572</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1.507</t>
+          <t>1.438</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>2.010</t>
+          <t>1.910</t>
         </is>
       </c>
       <c r="F23" t="b">
@@ -5578,17 +5578,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1.1971</t>
+          <t>1.1265</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>0.937</t>
+          <t>0.886</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.529</t>
+          <t>1.433</t>
         </is>
       </c>
       <c r="F24" t="b">
@@ -5619,17 +5619,17 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.2749</t>
+          <t>0.2626</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>0.164</t>
+          <t>0.157</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>0.462</t>
+          <t>0.440</t>
         </is>
       </c>
       <c r="F25" t="b">

</xml_diff>

<commit_message>
check in after running sim and boostrap; before time series
</commit_message>
<xml_diff>
--- a/data/Czech/KCOR_summary.xlsx
+++ b/data/Czech/KCOR_summary.xlsx
@@ -581,17 +581,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.9509</t>
+          <t>0.9563</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.875</t>
+          <t>0.879</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>1.034</t>
+          <t>1.040</t>
         </is>
       </c>
       <c r="F5" t="b">
@@ -622,17 +622,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.9581</t>
+          <t>0.9675</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.920</t>
+          <t>0.929</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.998</t>
+          <t>1.008</t>
         </is>
       </c>
       <c r="F6" t="b">
@@ -663,17 +663,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1.3659</t>
+          <t>1.3752</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.325</t>
+          <t>1.334</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.408</t>
+          <t>1.418</t>
         </is>
       </c>
       <c r="F7" t="b">
@@ -704,17 +704,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1.4484</t>
+          <t>1.4619</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.339</t>
+          <t>1.351</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.567</t>
+          <t>1.582</t>
         </is>
       </c>
       <c r="F8" t="b">
@@ -745,17 +745,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.2750</t>
+          <t>1.2838</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.101</t>
+          <t>1.109</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.476</t>
+          <t>1.487</t>
         </is>
       </c>
       <c r="F9" t="b">
@@ -786,17 +786,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2.8393</t>
+          <t>2.8803</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2.230</t>
+          <t>2.262</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>3.616</t>
+          <t>3.668</t>
         </is>
       </c>
       <c r="F10" t="b">
@@ -868,7 +868,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2.2365</t>
+          <t>2.2377</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -878,7 +878,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>3.751</t>
+          <t>3.753</t>
         </is>
       </c>
       <c r="F12" t="b">
@@ -909,7 +909,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>12.4845</t>
+          <t>12.4847</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -1025,17 +1025,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>1.2700</t>
+          <t>1.2787</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>1.216</t>
+          <t>1.224</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.327</t>
+          <t>1.336</t>
         </is>
       </c>
       <c r="F17" t="b">
@@ -1066,17 +1066,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.3886</t>
+          <t>1.4037</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1.355</t>
+          <t>1.369</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.423</t>
+          <t>1.439</t>
         </is>
       </c>
       <c r="F18" t="b">
@@ -1107,17 +1107,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1.4243</t>
+          <t>1.4339</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.371</t>
+          <t>1.380</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.480</t>
+          <t>1.490</t>
         </is>
       </c>
       <c r="F19" t="b">
@@ -1148,17 +1148,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1.1997</t>
+          <t>1.1758</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.119</t>
+          <t>1.094</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.286</t>
+          <t>1.263</t>
         </is>
       </c>
       <c r="F20" t="b">
@@ -1189,17 +1189,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.1567</t>
+          <t>1.1614</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.001</t>
+          <t>1.004</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.337</t>
+          <t>1.343</t>
         </is>
       </c>
       <c r="F21" t="b">
@@ -1230,17 +1230,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.0500</t>
+          <t>1.0652</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.827</t>
+          <t>0.838</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.334</t>
+          <t>1.353</t>
         </is>
       </c>
       <c r="F22" t="b">
@@ -1312,7 +1312,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1.1881</t>
+          <t>1.1887</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -1322,7 +1322,7 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>1.991</t>
+          <t>1.992</t>
         </is>
       </c>
       <c r="F24" t="b">
@@ -1353,7 +1353,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2.2478</t>
+          <t>2.2479</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1363,7 +1363,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>16.031</t>
+          <t>16.032</t>
         </is>
       </c>
       <c r="F25" t="b">
@@ -1469,17 +1469,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1.3356</t>
+          <t>1.3372</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1.226</t>
+          <t>1.227</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.455</t>
+          <t>1.457</t>
         </is>
       </c>
       <c r="F29" t="b">
@@ -1510,17 +1510,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1.4492</t>
+          <t>1.4509</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1.389</t>
+          <t>1.391</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.512</t>
+          <t>1.514</t>
         </is>
       </c>
       <c r="F30" t="b">
@@ -1592,17 +1592,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.8283</t>
+          <t>0.8042</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.747</t>
+          <t>0.724</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0.918</t>
+          <t>0.893</t>
         </is>
       </c>
       <c r="F32" t="b">
@@ -1633,17 +1633,17 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>0.9072</t>
+          <t>0.9047</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>0.740</t>
+          <t>0.738</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>1.112</t>
+          <t>1.109</t>
         </is>
       </c>
       <c r="F33" t="b">
@@ -2003,17 +2003,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.7497</t>
+          <t>0.7542</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0.682</t>
+          <t>0.686</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.824</t>
+          <t>0.829</t>
         </is>
       </c>
       <c r="F5" t="b">
@@ -2044,17 +2044,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.9737</t>
+          <t>0.9887</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.926</t>
+          <t>0.940</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>1.024</t>
+          <t>1.040</t>
         </is>
       </c>
       <c r="F6" t="b">
@@ -2085,17 +2085,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>1.0447</t>
+          <t>1.0755</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>1.010</t>
+          <t>1.040</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>1.080</t>
+          <t>1.112</t>
         </is>
       </c>
       <c r="F7" t="b">
@@ -2126,17 +2126,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1.4261</t>
+          <t>1.4794</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.379</t>
+          <t>1.430</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.475</t>
+          <t>1.530</t>
         </is>
       </c>
       <c r="F8" t="b">
@@ -2167,17 +2167,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.3663</t>
+          <t>1.4182</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.286</t>
+          <t>1.335</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.451</t>
+          <t>1.507</t>
         </is>
       </c>
       <c r="F9" t="b">
@@ -2208,17 +2208,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1.1983</t>
+          <t>1.2390</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.066</t>
+          <t>1.102</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.347</t>
+          <t>1.393</t>
         </is>
       </c>
       <c r="F10" t="b">
@@ -2249,17 +2249,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1.1406</t>
+          <t>1.1591</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>0.897</t>
+          <t>0.911</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>1.451</t>
+          <t>1.475</t>
         </is>
       </c>
       <c r="F11" t="b">
@@ -2290,7 +2290,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1.0243</t>
+          <t>1.0244</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -2300,7 +2300,7 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>1.689</t>
+          <t>1.690</t>
         </is>
       </c>
       <c r="F12" t="b">
@@ -2331,7 +2331,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>7.2631</t>
+          <t>7.2633</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2447,17 +2447,17 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>0.9628</t>
+          <t>0.9696</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>0.922</t>
+          <t>0.928</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1.005</t>
+          <t>1.013</t>
         </is>
       </c>
       <c r="F17" t="b">
@@ -2488,17 +2488,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>1.0045</t>
+          <t>1.0199</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.980</t>
+          <t>0.995</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>1.029</t>
+          <t>1.045</t>
         </is>
       </c>
       <c r="F18" t="b">
@@ -2529,17 +2529,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1.2221</t>
+          <t>1.2582</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.192</t>
+          <t>1.226</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.253</t>
+          <t>1.291</t>
         </is>
       </c>
       <c r="F19" t="b">
@@ -2570,17 +2570,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1.0457</t>
+          <t>1.0602</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.996</t>
+          <t>1.009</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.098</t>
+          <t>1.114</t>
         </is>
       </c>
       <c r="F20" t="b">
@@ -2611,17 +2611,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.1845</t>
+          <t>1.2295</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.078</t>
+          <t>1.119</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.301</t>
+          <t>1.351</t>
         </is>
       </c>
       <c r="F21" t="b">
@@ -2652,17 +2652,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.9918</t>
+          <t>1.0255</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.853</t>
+          <t>0.881</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.154</t>
+          <t>1.193</t>
         </is>
       </c>
       <c r="F22" t="b">
@@ -2693,17 +2693,17 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2.6376</t>
+          <t>2.6803</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>2.064</t>
+          <t>2.097</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>3.371</t>
+          <t>3.427</t>
         </is>
       </c>
       <c r="F23" t="b">
@@ -2734,7 +2734,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.8501</t>
+          <t>0.8502</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -2775,7 +2775,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>6.7260</t>
+          <t>6.7262</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -2785,7 +2785,7 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>13.110</t>
+          <t>13.111</t>
         </is>
       </c>
       <c r="F25" t="b">
@@ -2891,17 +2891,17 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>1.2843</t>
+          <t>1.2856</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>1.169</t>
+          <t>1.170</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>1.411</t>
+          <t>1.413</t>
         </is>
       </c>
       <c r="F29" t="b">
@@ -3014,17 +3014,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>0.7332</t>
+          <t>0.7166</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>0.695</t>
+          <t>0.679</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>0.773</t>
+          <t>0.757</t>
         </is>
       </c>
       <c r="F32" t="b">
@@ -3466,17 +3466,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.8905</t>
+          <t>0.9019</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.843</t>
+          <t>0.853</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.941</t>
+          <t>0.953</t>
         </is>
       </c>
       <c r="F6" t="b">
@@ -3507,17 +3507,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.8708</t>
+          <t>0.9000</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.834</t>
+          <t>0.862</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.909</t>
+          <t>0.940</t>
         </is>
       </c>
       <c r="F7" t="b">
@@ -3548,17 +3548,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1.0864</t>
+          <t>1.1401</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.043</t>
+          <t>1.094</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>1.131</t>
+          <t>1.188</t>
         </is>
       </c>
       <c r="F8" t="b">
@@ -3589,17 +3589,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>1.0885</t>
+          <t>1.1413</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1.027</t>
+          <t>1.076</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.154</t>
+          <t>1.211</t>
         </is>
       </c>
       <c r="F9" t="b">
@@ -3630,17 +3630,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1.1995</t>
+          <t>1.2440</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>1.098</t>
+          <t>1.138</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.310</t>
+          <t>1.360</t>
         </is>
       </c>
       <c r="F10" t="b">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>1.135</t>
+          <t>1.136</t>
         </is>
       </c>
       <c r="F13" t="b">
@@ -3910,17 +3910,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.9543</t>
+          <t>0.9696</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.931</t>
+          <t>0.946</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0.978</t>
+          <t>0.994</t>
         </is>
       </c>
       <c r="F18" t="b">
@@ -3951,17 +3951,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1.0657</t>
+          <t>1.1030</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>1.040</t>
+          <t>1.076</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>1.092</t>
+          <t>1.130</t>
         </is>
       </c>
       <c r="F19" t="b">
@@ -3992,17 +3992,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>1.2876</t>
+          <t>1.3513</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>1.245</t>
+          <t>1.306</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>1.332</t>
+          <t>1.399</t>
         </is>
       </c>
       <c r="F20" t="b">
@@ -4033,17 +4033,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.0379</t>
+          <t>1.0883</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0.969</t>
+          <t>1.016</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.112</t>
+          <t>1.166</t>
         </is>
       </c>
       <c r="F21" t="b">
@@ -4074,17 +4074,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.0787</t>
+          <t>1.1188</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.964</t>
+          <t>1.000</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.207</t>
+          <t>1.252</t>
         </is>
       </c>
       <c r="F22" t="b">
@@ -4197,7 +4197,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>0.9564</t>
+          <t>0.9565</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -4354,17 +4354,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1.0717</t>
+          <t>1.0751</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1.015</t>
+          <t>1.018</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.132</t>
+          <t>1.135</t>
         </is>
       </c>
       <c r="F30" t="b">
@@ -4395,17 +4395,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>1.2238</t>
+          <t>1.2256</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>1.172</t>
+          <t>1.173</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1.278</t>
+          <t>1.280</t>
         </is>
       </c>
       <c r="F31" t="b">
@@ -4888,17 +4888,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.6796</t>
+          <t>0.6861</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>0.630</t>
+          <t>0.636</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0.733</t>
+          <t>0.741</t>
         </is>
       </c>
       <c r="F6" t="b">
@@ -4929,17 +4929,17 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.5852</t>
+          <t>0.6071</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.544</t>
+          <t>0.564</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0.630</t>
+          <t>0.654</t>
         </is>
       </c>
       <c r="F7" t="b">
@@ -4970,17 +4970,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.6148</t>
+          <t>0.6494</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>0.569</t>
+          <t>0.601</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0.665</t>
+          <t>0.702</t>
         </is>
       </c>
       <c r="F8" t="b">
@@ -5011,17 +5011,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.9279</t>
+          <t>0.9741</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>0.831</t>
+          <t>0.872</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>1.036</t>
+          <t>1.088</t>
         </is>
       </c>
       <c r="F9" t="b">
@@ -5052,17 +5052,17 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>1.0309</t>
+          <t>1.0766</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>0.891</t>
+          <t>0.929</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>1.193</t>
+          <t>1.247</t>
         </is>
       </c>
       <c r="F10" t="b">
@@ -5332,17 +5332,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>0.8475</t>
+          <t>0.8582</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>0.826</t>
+          <t>0.837</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>0.869</t>
+          <t>0.880</t>
         </is>
       </c>
       <c r="F18" t="b">
@@ -5373,17 +5373,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.9278</t>
+          <t>0.9625</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>0.906</t>
+          <t>0.940</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0.950</t>
+          <t>0.986</t>
         </is>
       </c>
       <c r="F19" t="b">
@@ -5414,17 +5414,17 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>0.9452</t>
+          <t>0.9983</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>0.917</t>
+          <t>0.968</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>0.974</t>
+          <t>1.030</t>
         </is>
       </c>
       <c r="F20" t="b">
@@ -5455,17 +5455,17 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>1.2347</t>
+          <t>1.2962</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>1.176</t>
+          <t>1.233</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>1.296</t>
+          <t>1.362</t>
         </is>
       </c>
       <c r="F21" t="b">
@@ -5496,17 +5496,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1.0700</t>
+          <t>1.1174</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.992</t>
+          <t>1.035</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>1.154</t>
+          <t>1.206</t>
         </is>
       </c>
       <c r="F22" t="b">
@@ -5776,17 +5776,17 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>1.2471</t>
+          <t>1.2509</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>1.157</t>
+          <t>1.160</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>1.344</t>
+          <t>1.349</t>
         </is>
       </c>
       <c r="F30" t="b">

</xml_diff>